<commit_message>
feat: redesign admin panel + add Comercial/Pricing to internal contacts
- Admin panel (dashboard + detail view): navy header bars, grey page background,
  corporate color scheme (navy #1B2A4A, red #C8102E), DetailsSection ghost numbers
- Add Comercial and Pricing/Inside Sale to ContactosInternosEditor (rows 32-33 in Excel)
- Split AREAS_CONTACTO_INTERNOS (6) from AREAS_CONTACTO (4); update schemas, defaults,
  migrator, store, excelExport and PATCH route validator accordingly
- Migration function prepends empty Comercial/Pricing rows to legacy 4-row records

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/formats/formato_SOP_old.xlsx
+++ b/formats/formato_SOP_old.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -1156,6 +1156,271 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -1164,273 +1429,8 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -1974,60 +1974,60 @@
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="2:15" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="42" t="e" vm="1">
+      <c r="B2" s="74" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="43" t="s">
+      <c r="C2" s="74"/>
+      <c r="D2" s="75" t="s">
         <v>124</v>
       </c>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="45" t="s">
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
+      <c r="I2" s="76"/>
+      <c r="J2" s="76"/>
+      <c r="K2" s="76"/>
+      <c r="L2" s="76"/>
+      <c r="M2" s="76"/>
+      <c r="N2" s="77" t="s">
         <v>104</v>
       </c>
-      <c r="O2" s="46"/>
+      <c r="O2" s="78"/>
     </row>
     <row r="3" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="47"/>
+      <c r="B3" s="79"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="79"/>
+      <c r="L3" s="79"/>
+      <c r="M3" s="79"/>
+      <c r="N3" s="79"/>
+      <c r="O3" s="79"/>
     </row>
     <row r="4" spans="2:15" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="37"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="43"/>
+      <c r="J4" s="43"/>
+      <c r="K4" s="43"/>
+      <c r="L4" s="43"/>
+      <c r="M4" s="43"/>
+      <c r="N4" s="43"/>
+      <c r="O4" s="44"/>
     </row>
     <row r="5" spans="2:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="13" t="s">
@@ -2036,152 +2036,152 @@
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
-      <c r="F5" s="74" t="s">
+      <c r="F5" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="75"/>
-      <c r="H5" s="76"/>
-      <c r="I5" s="77" t="s">
+      <c r="G5" s="62"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="64" t="s">
         <v>142</v>
       </c>
-      <c r="J5" s="78"/>
-      <c r="K5" s="79"/>
-      <c r="L5" s="48" t="s">
+      <c r="J5" s="65"/>
+      <c r="K5" s="66"/>
+      <c r="L5" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="27"/>
     </row>
     <row r="6" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="B6" s="15"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="67"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="91"/>
-      <c r="L6" s="55"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="26"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="27"/>
     </row>
     <row r="7" spans="2:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="87" t="s">
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="88"/>
-      <c r="H7" s="88"/>
-      <c r="I7" s="88"/>
-      <c r="J7" s="88"/>
-      <c r="K7" s="88"/>
-      <c r="L7" s="88"/>
-      <c r="M7" s="88"/>
-      <c r="N7" s="88"/>
-      <c r="O7" s="89"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="20"/>
     </row>
     <row r="8" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B8" s="55"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="90"/>
-      <c r="G8" s="68"/>
-      <c r="H8" s="68"/>
-      <c r="I8" s="68"/>
-      <c r="J8" s="68"/>
-      <c r="K8" s="68"/>
-      <c r="L8" s="68"/>
-      <c r="M8" s="68"/>
-      <c r="N8" s="68"/>
-      <c r="O8" s="91"/>
+      <c r="B8" s="49"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="23"/>
     </row>
     <row r="9" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="48" t="s">
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="28"/>
-      <c r="L9" s="26"/>
-      <c r="M9" s="48" t="s">
+      <c r="K9" s="26"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="28" t="s">
         <v>129</v>
       </c>
-      <c r="N9" s="28"/>
-      <c r="O9" s="26"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="27"/>
     </row>
     <row r="10" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B10" s="55"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="55"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="55"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="26"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="49"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="27"/>
     </row>
     <row r="11" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="57"/>
-      <c r="D11" s="57"/>
-      <c r="E11" s="57"/>
-      <c r="F11" s="57"/>
-      <c r="G11" s="57"/>
-      <c r="H11" s="58"/>
-      <c r="I11" s="59" t="s">
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="70"/>
+      <c r="I11" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="57"/>
-      <c r="K11" s="57"/>
-      <c r="L11" s="57"/>
-      <c r="M11" s="57"/>
-      <c r="N11" s="57"/>
-      <c r="O11" s="60"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="69"/>
+      <c r="L11" s="69"/>
+      <c r="M11" s="69"/>
+      <c r="N11" s="69"/>
+      <c r="O11" s="72"/>
     </row>
     <row r="12" spans="2:15" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="83" t="s">
         <v>131</v>
       </c>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="49" t="s">
+      <c r="C12" s="81"/>
+      <c r="D12" s="81"/>
+      <c r="E12" s="81"/>
+      <c r="F12" s="81"/>
+      <c r="G12" s="81"/>
+      <c r="H12" s="81"/>
+      <c r="I12" s="80" t="s">
         <v>133</v>
       </c>
-      <c r="J12" s="33"/>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
-      <c r="N12" s="33"/>
-      <c r="O12" s="50"/>
+      <c r="J12" s="81"/>
+      <c r="K12" s="81"/>
+      <c r="L12" s="81"/>
+      <c r="M12" s="81"/>
+      <c r="N12" s="81"/>
+      <c r="O12" s="82"/>
     </row>
     <row r="13" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="5"/>
@@ -2200,146 +2200,146 @@
       <c r="O13" s="5"/>
     </row>
     <row r="14" spans="2:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="37"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="43"/>
+      <c r="L14" s="43"/>
+      <c r="M14" s="43"/>
+      <c r="N14" s="43"/>
+      <c r="O14" s="44"/>
     </row>
     <row r="15" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="48" t="s">
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
-      <c r="L15" s="28"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="28"/>
-      <c r="O15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="26"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="27"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="27"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="61"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="61"/>
-      <c r="H16" s="62"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="61"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61"/>
-      <c r="N16" s="61"/>
-      <c r="O16" s="62"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35"/>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35"/>
+      <c r="N16" s="35"/>
+      <c r="O16" s="36"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="70"/>
-      <c r="C17" s="71"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="71"/>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71"/>
-      <c r="H17" s="72"/>
-      <c r="I17" s="70"/>
-      <c r="J17" s="71"/>
-      <c r="K17" s="71"/>
-      <c r="L17" s="71"/>
-      <c r="M17" s="71"/>
-      <c r="N17" s="71"/>
-      <c r="O17" s="72"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="51"/>
+      <c r="D17" s="51"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="51"/>
+      <c r="H17" s="48"/>
+      <c r="I17" s="47"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="51"/>
+      <c r="L17" s="51"/>
+      <c r="M17" s="51"/>
+      <c r="N17" s="51"/>
+      <c r="O17" s="48"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="70"/>
-      <c r="C18" s="71"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="71"/>
-      <c r="F18" s="71"/>
-      <c r="G18" s="71"/>
-      <c r="H18" s="72"/>
-      <c r="I18" s="70"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="71"/>
-      <c r="L18" s="71"/>
-      <c r="M18" s="71"/>
-      <c r="N18" s="71"/>
-      <c r="O18" s="72"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="51"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="51"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="47"/>
+      <c r="J18" s="51"/>
+      <c r="K18" s="51"/>
+      <c r="L18" s="51"/>
+      <c r="M18" s="51"/>
+      <c r="N18" s="51"/>
+      <c r="O18" s="48"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="63"/>
-      <c r="C19" s="64"/>
-      <c r="D19" s="64"/>
-      <c r="E19" s="64"/>
-      <c r="F19" s="64"/>
-      <c r="G19" s="64"/>
-      <c r="H19" s="65"/>
-      <c r="I19" s="63"/>
-      <c r="J19" s="64"/>
-      <c r="K19" s="64"/>
-      <c r="L19" s="64"/>
-      <c r="M19" s="64"/>
-      <c r="N19" s="64"/>
-      <c r="O19" s="65"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="39"/>
+      <c r="I19" s="37"/>
+      <c r="J19" s="38"/>
+      <c r="K19" s="38"/>
+      <c r="L19" s="38"/>
+      <c r="M19" s="38"/>
+      <c r="N19" s="38"/>
+      <c r="O19" s="39"/>
     </row>
     <row r="20" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B20" s="48" t="s">
+      <c r="B20" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="48" t="s">
+      <c r="C20" s="26"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="F20" s="28"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="48" t="s">
+      <c r="F20" s="26"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="84" t="s">
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="60" t="s">
         <v>150</v>
       </c>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="27"/>
     </row>
     <row r="21" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B21" s="27"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="26"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="25"/>
+      <c r="M21" s="26"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="27"/>
     </row>
     <row r="22" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="5"/>
@@ -2358,370 +2358,370 @@
       <c r="O22" s="5"/>
     </row>
     <row r="23" spans="2:15" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="82"/>
-      <c r="D23" s="82"/>
-      <c r="E23" s="82"/>
-      <c r="F23" s="82"/>
-      <c r="G23" s="82"/>
-      <c r="H23" s="82"/>
-      <c r="I23" s="82"/>
-      <c r="J23" s="82"/>
-      <c r="K23" s="82"/>
-      <c r="L23" s="82"/>
-      <c r="M23" s="82"/>
-      <c r="N23" s="82"/>
-      <c r="O23" s="83"/>
+      <c r="C23" s="58"/>
+      <c r="D23" s="58"/>
+      <c r="E23" s="58"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
+      <c r="J23" s="58"/>
+      <c r="K23" s="58"/>
+      <c r="L23" s="58"/>
+      <c r="M23" s="58"/>
+      <c r="N23" s="58"/>
+      <c r="O23" s="59"/>
     </row>
     <row r="24" spans="2:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="30"/>
-      <c r="K24" s="30"/>
-      <c r="L24" s="30"/>
-      <c r="M24" s="30"/>
-      <c r="N24" s="30"/>
-      <c r="O24" s="31"/>
+      <c r="C24" s="85"/>
+      <c r="D24" s="85"/>
+      <c r="E24" s="85"/>
+      <c r="F24" s="85"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="85"/>
+      <c r="I24" s="85"/>
+      <c r="J24" s="85"/>
+      <c r="K24" s="85"/>
+      <c r="L24" s="85"/>
+      <c r="M24" s="85"/>
+      <c r="N24" s="85"/>
+      <c r="O24" s="86"/>
     </row>
     <row r="25" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="87" t="s">
         <v>146</v>
       </c>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="30"/>
-      <c r="K25" s="40" t="s">
+      <c r="C25" s="85"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="85"/>
+      <c r="F25" s="85"/>
+      <c r="G25" s="85"/>
+      <c r="H25" s="85"/>
+      <c r="I25" s="85"/>
+      <c r="J25" s="85"/>
+      <c r="K25" s="84" t="s">
         <v>145</v>
       </c>
-      <c r="L25" s="30"/>
-      <c r="M25" s="30"/>
-      <c r="N25" s="30"/>
-      <c r="O25" s="31"/>
+      <c r="L25" s="85"/>
+      <c r="M25" s="85"/>
+      <c r="N25" s="85"/>
+      <c r="O25" s="86"/>
     </row>
     <row r="26" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B26" s="38" t="s">
+      <c r="B26" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="26"/>
-      <c r="D26" s="38" t="s">
+      <c r="C26" s="27"/>
+      <c r="D26" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="26"/>
+      <c r="E26" s="27"/>
       <c r="F26" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G26" s="38" t="s">
+      <c r="G26" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="H26" s="26"/>
-      <c r="I26" s="38" t="s">
+      <c r="H26" s="27"/>
+      <c r="I26" s="29" t="s">
         <v>166</v>
       </c>
-      <c r="J26" s="26"/>
-      <c r="K26" s="38" t="s">
+      <c r="J26" s="27"/>
+      <c r="K26" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="L26" s="26"/>
+      <c r="L26" s="27"/>
       <c r="M26" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="N26" s="38" t="s">
+      <c r="N26" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="O26" s="26"/>
+      <c r="O26" s="27"/>
     </row>
     <row r="27" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B27" s="39" t="s">
+      <c r="B27" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C27" s="26"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="26"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="27"/>
       <c r="F27" s="4"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="27"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="26"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="27"/>
       <c r="M27" s="4"/>
-      <c r="N27" s="27"/>
-      <c r="O27" s="26"/>
+      <c r="N27" s="25"/>
+      <c r="O27" s="27"/>
     </row>
     <row r="28" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B28" s="39" t="s">
+      <c r="B28" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="C28" s="26"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="26"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="27"/>
       <c r="F28" s="4"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="27"/>
-      <c r="J28" s="26"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="26"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="27"/>
       <c r="M28" s="4"/>
-      <c r="N28" s="27"/>
-      <c r="O28" s="26"/>
+      <c r="N28" s="25"/>
+      <c r="O28" s="27"/>
     </row>
     <row r="29" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B29" s="39" t="s">
+      <c r="B29" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="C29" s="26"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="26"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="4"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="26"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="27"/>
       <c r="M29" s="4"/>
-      <c r="N29" s="27"/>
-      <c r="O29" s="26"/>
+      <c r="N29" s="25"/>
+      <c r="O29" s="27"/>
     </row>
     <row r="30" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B30" s="39" t="s">
+      <c r="B30" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="C30" s="26"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="26"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="27"/>
       <c r="F30" s="4"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="26"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="26"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="27"/>
       <c r="M30" s="4"/>
-      <c r="N30" s="27"/>
-      <c r="O30" s="26"/>
+      <c r="N30" s="25"/>
+      <c r="O30" s="27"/>
     </row>
     <row r="31" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B31" s="39"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="26"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="27"/>
       <c r="F31" s="4"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="26"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="26"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="27"/>
       <c r="M31" s="4"/>
-      <c r="N31" s="27"/>
-      <c r="O31" s="26"/>
+      <c r="N31" s="25"/>
+      <c r="O31" s="27"/>
     </row>
     <row r="32" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B32" s="39"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="26"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="27"/>
       <c r="F32" s="4"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="27"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="26"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="27"/>
       <c r="M32" s="4"/>
-      <c r="N32" s="27"/>
-      <c r="O32" s="26"/>
+      <c r="N32" s="25"/>
+      <c r="O32" s="27"/>
     </row>
     <row r="33" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="87" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="30"/>
-      <c r="M33" s="30"/>
-      <c r="N33" s="30"/>
-      <c r="O33" s="31"/>
+      <c r="C33" s="85"/>
+      <c r="D33" s="85"/>
+      <c r="E33" s="85"/>
+      <c r="F33" s="85"/>
+      <c r="G33" s="85"/>
+      <c r="H33" s="85"/>
+      <c r="I33" s="85"/>
+      <c r="J33" s="85"/>
+      <c r="K33" s="85"/>
+      <c r="L33" s="85"/>
+      <c r="M33" s="85"/>
+      <c r="N33" s="85"/>
+      <c r="O33" s="86"/>
     </row>
     <row r="34" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="87" t="s">
         <v>146</v>
       </c>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
-      <c r="J34" s="30"/>
-      <c r="K34" s="40" t="s">
+      <c r="C34" s="85"/>
+      <c r="D34" s="85"/>
+      <c r="E34" s="85"/>
+      <c r="F34" s="85"/>
+      <c r="G34" s="85"/>
+      <c r="H34" s="85"/>
+      <c r="I34" s="85"/>
+      <c r="J34" s="85"/>
+      <c r="K34" s="84" t="s">
         <v>145</v>
       </c>
-      <c r="L34" s="30"/>
-      <c r="M34" s="30"/>
-      <c r="N34" s="30"/>
-      <c r="O34" s="31"/>
+      <c r="L34" s="85"/>
+      <c r="M34" s="85"/>
+      <c r="N34" s="85"/>
+      <c r="O34" s="86"/>
     </row>
     <row r="35" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B35" s="38" t="s">
+      <c r="B35" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="26"/>
-      <c r="D35" s="38" t="s">
+      <c r="C35" s="27"/>
+      <c r="D35" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="E35" s="26"/>
+      <c r="E35" s="27"/>
       <c r="F35" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G35" s="38" t="s">
+      <c r="G35" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="H35" s="26"/>
-      <c r="I35" s="38" t="s">
+      <c r="H35" s="27"/>
+      <c r="I35" s="29" t="s">
         <v>166</v>
       </c>
-      <c r="J35" s="26"/>
-      <c r="K35" s="38" t="s">
+      <c r="J35" s="27"/>
+      <c r="K35" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="L35" s="26"/>
+      <c r="L35" s="27"/>
       <c r="M35" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="N35" s="38" t="s">
+      <c r="N35" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="O35" s="26"/>
+      <c r="O35" s="27"/>
     </row>
     <row r="36" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B36" s="39" t="s">
+      <c r="B36" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C36" s="26"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="26"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="27"/>
       <c r="F36" s="4"/>
-      <c r="G36" s="27"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="27"/>
-      <c r="J36" s="26"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="26"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="25"/>
+      <c r="L36" s="27"/>
       <c r="M36" s="4"/>
-      <c r="N36" s="27"/>
-      <c r="O36" s="26"/>
+      <c r="N36" s="25"/>
+      <c r="O36" s="27"/>
     </row>
     <row r="37" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B37" s="39" t="s">
+      <c r="B37" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="C37" s="26"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="26"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="27"/>
       <c r="F37" s="4"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="26"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="26"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="25"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="25"/>
+      <c r="L37" s="27"/>
       <c r="M37" s="4"/>
-      <c r="N37" s="27"/>
-      <c r="O37" s="26"/>
+      <c r="N37" s="25"/>
+      <c r="O37" s="27"/>
     </row>
     <row r="38" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B38" s="39" t="s">
+      <c r="B38" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="C38" s="26"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="26"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="27"/>
       <c r="F38" s="4"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="26"/>
-      <c r="K38" s="27"/>
-      <c r="L38" s="26"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="25"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="25"/>
+      <c r="L38" s="27"/>
       <c r="M38" s="4"/>
-      <c r="N38" s="27"/>
-      <c r="O38" s="26"/>
+      <c r="N38" s="25"/>
+      <c r="O38" s="27"/>
     </row>
     <row r="39" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B39" s="39" t="s">
+      <c r="B39" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="C39" s="26"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="26"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="25"/>
+      <c r="E39" s="27"/>
       <c r="F39" s="4"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="27"/>
-      <c r="J39" s="26"/>
-      <c r="K39" s="27"/>
-      <c r="L39" s="26"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="25"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="25"/>
+      <c r="L39" s="27"/>
       <c r="M39" s="4"/>
-      <c r="N39" s="27"/>
-      <c r="O39" s="26"/>
+      <c r="N39" s="25"/>
+      <c r="O39" s="27"/>
     </row>
     <row r="40" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B40" s="39"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="26"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="25"/>
+      <c r="E40" s="27"/>
       <c r="F40" s="4"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="26"/>
-      <c r="K40" s="27"/>
-      <c r="L40" s="26"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="25"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="25"/>
+      <c r="L40" s="27"/>
       <c r="M40" s="4"/>
-      <c r="N40" s="27"/>
-      <c r="O40" s="26"/>
+      <c r="N40" s="25"/>
+      <c r="O40" s="27"/>
     </row>
     <row r="41" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B41" s="39"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="26"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="25"/>
+      <c r="E41" s="27"/>
       <c r="F41" s="4"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="26"/>
-      <c r="K41" s="27"/>
-      <c r="L41" s="26"/>
+      <c r="G41" s="25"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="25"/>
+      <c r="J41" s="27"/>
+      <c r="K41" s="25"/>
+      <c r="L41" s="27"/>
       <c r="M41" s="4"/>
-      <c r="N41" s="27"/>
-      <c r="O41" s="26"/>
+      <c r="N41" s="25"/>
+      <c r="O41" s="27"/>
     </row>
     <row r="42" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="5"/>
@@ -2740,96 +2740,96 @@
       <c r="O42" s="5"/>
     </row>
     <row r="43" spans="2:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="35" t="s">
+      <c r="B43" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C43" s="36"/>
-      <c r="D43" s="36"/>
-      <c r="E43" s="36"/>
-      <c r="F43" s="36"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="36"/>
-      <c r="I43" s="36"/>
-      <c r="J43" s="36"/>
-      <c r="K43" s="36"/>
-      <c r="L43" s="36"/>
-      <c r="M43" s="36"/>
-      <c r="N43" s="36"/>
-      <c r="O43" s="37"/>
+      <c r="C43" s="43"/>
+      <c r="D43" s="43"/>
+      <c r="E43" s="43"/>
+      <c r="F43" s="43"/>
+      <c r="G43" s="43"/>
+      <c r="H43" s="43"/>
+      <c r="I43" s="43"/>
+      <c r="J43" s="43"/>
+      <c r="K43" s="43"/>
+      <c r="L43" s="43"/>
+      <c r="M43" s="43"/>
+      <c r="N43" s="43"/>
+      <c r="O43" s="44"/>
     </row>
     <row r="44" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B44" s="66" t="s">
+      <c r="B44" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="28"/>
-      <c r="I44" s="28"/>
-      <c r="J44" s="28"/>
-      <c r="K44" s="28"/>
-      <c r="L44" s="28"/>
-      <c r="M44" s="28"/>
-      <c r="N44" s="28"/>
-      <c r="O44" s="26"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="26"/>
+      <c r="F44" s="26"/>
+      <c r="G44" s="26"/>
+      <c r="H44" s="26"/>
+      <c r="I44" s="26"/>
+      <c r="J44" s="26"/>
+      <c r="K44" s="26"/>
+      <c r="L44" s="26"/>
+      <c r="M44" s="26"/>
+      <c r="N44" s="26"/>
+      <c r="O44" s="27"/>
     </row>
     <row r="45" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B45" s="48" t="s">
+      <c r="B45" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="C45" s="28"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="48" t="s">
+      <c r="C45" s="26"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="F45" s="28"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="48" t="s">
+      <c r="F45" s="26"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="I45" s="28"/>
-      <c r="J45" s="28"/>
-      <c r="K45" s="26"/>
-      <c r="L45" s="48" t="s">
+      <c r="I45" s="26"/>
+      <c r="J45" s="26"/>
+      <c r="K45" s="27"/>
+      <c r="L45" s="28" t="s">
         <v>130</v>
       </c>
-      <c r="M45" s="28"/>
-      <c r="N45" s="28"/>
-      <c r="O45" s="26"/>
+      <c r="M45" s="26"/>
+      <c r="N45" s="26"/>
+      <c r="O45" s="27"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B46" s="27"/>
-      <c r="C46" s="61"/>
-      <c r="D46" s="62"/>
-      <c r="E46" s="27"/>
-      <c r="F46" s="61"/>
-      <c r="G46" s="62"/>
-      <c r="H46" s="27"/>
-      <c r="I46" s="61"/>
-      <c r="J46" s="61"/>
-      <c r="K46" s="62"/>
-      <c r="L46" s="27"/>
-      <c r="M46" s="61"/>
-      <c r="N46" s="61"/>
-      <c r="O46" s="62"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="25"/>
+      <c r="F46" s="35"/>
+      <c r="G46" s="36"/>
+      <c r="H46" s="25"/>
+      <c r="I46" s="35"/>
+      <c r="J46" s="35"/>
+      <c r="K46" s="36"/>
+      <c r="L46" s="25"/>
+      <c r="M46" s="35"/>
+      <c r="N46" s="35"/>
+      <c r="O46" s="36"/>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B47" s="63"/>
-      <c r="C47" s="64"/>
-      <c r="D47" s="65"/>
-      <c r="E47" s="63"/>
-      <c r="F47" s="64"/>
-      <c r="G47" s="65"/>
-      <c r="H47" s="63"/>
-      <c r="I47" s="64"/>
-      <c r="J47" s="64"/>
-      <c r="K47" s="65"/>
-      <c r="L47" s="63"/>
-      <c r="M47" s="64"/>
-      <c r="N47" s="64"/>
-      <c r="O47" s="65"/>
+      <c r="B47" s="37"/>
+      <c r="C47" s="38"/>
+      <c r="D47" s="39"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="38"/>
+      <c r="G47" s="39"/>
+      <c r="H47" s="37"/>
+      <c r="I47" s="38"/>
+      <c r="J47" s="38"/>
+      <c r="K47" s="39"/>
+      <c r="L47" s="37"/>
+      <c r="M47" s="38"/>
+      <c r="N47" s="38"/>
+      <c r="O47" s="39"/>
     </row>
     <row r="48" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="B48" s="5"/>
@@ -2848,202 +2848,202 @@
       <c r="O48" s="5"/>
     </row>
     <row r="49" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B49" s="66" t="s">
+      <c r="B49" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28"/>
-      <c r="F49" s="28"/>
-      <c r="G49" s="28"/>
-      <c r="H49" s="28"/>
-      <c r="I49" s="28"/>
-      <c r="J49" s="28"/>
-      <c r="K49" s="28"/>
-      <c r="L49" s="28"/>
-      <c r="M49" s="28"/>
-      <c r="N49" s="28"/>
-      <c r="O49" s="26"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="26"/>
+      <c r="I49" s="26"/>
+      <c r="J49" s="26"/>
+      <c r="K49" s="26"/>
+      <c r="L49" s="26"/>
+      <c r="M49" s="26"/>
+      <c r="N49" s="26"/>
+      <c r="O49" s="27"/>
     </row>
     <row r="50" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B50" s="48" t="s">
+      <c r="B50" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C50" s="28"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="48" t="s">
+      <c r="C50" s="26"/>
+      <c r="D50" s="27"/>
+      <c r="E50" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="F50" s="28"/>
-      <c r="G50" s="26"/>
-      <c r="H50" s="48" t="s">
+      <c r="F50" s="26"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="I50" s="28"/>
-      <c r="J50" s="28"/>
-      <c r="K50" s="26"/>
-      <c r="L50" s="48" t="s">
+      <c r="I50" s="26"/>
+      <c r="J50" s="26"/>
+      <c r="K50" s="27"/>
+      <c r="L50" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="M50" s="28"/>
-      <c r="N50" s="28"/>
-      <c r="O50" s="26"/>
+      <c r="M50" s="26"/>
+      <c r="N50" s="26"/>
+      <c r="O50" s="27"/>
     </row>
     <row r="51" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="27" t="s">
+      <c r="B51" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="C51" s="61"/>
-      <c r="D51" s="62"/>
-      <c r="E51" s="27" t="s">
+      <c r="C51" s="35"/>
+      <c r="D51" s="36"/>
+      <c r="E51" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="F51" s="61"/>
-      <c r="G51" s="62"/>
-      <c r="H51" s="27"/>
-      <c r="I51" s="61"/>
-      <c r="J51" s="61"/>
-      <c r="K51" s="62"/>
-      <c r="L51" s="27"/>
-      <c r="M51" s="61"/>
-      <c r="N51" s="61"/>
-      <c r="O51" s="62"/>
+      <c r="F51" s="35"/>
+      <c r="G51" s="36"/>
+      <c r="H51" s="25"/>
+      <c r="I51" s="35"/>
+      <c r="J51" s="35"/>
+      <c r="K51" s="36"/>
+      <c r="L51" s="25"/>
+      <c r="M51" s="35"/>
+      <c r="N51" s="35"/>
+      <c r="O51" s="36"/>
     </row>
     <row r="52" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="63"/>
-      <c r="C52" s="64"/>
-      <c r="D52" s="65"/>
-      <c r="E52" s="63"/>
-      <c r="F52" s="64"/>
-      <c r="G52" s="65"/>
-      <c r="H52" s="63"/>
-      <c r="I52" s="64"/>
-      <c r="J52" s="64"/>
-      <c r="K52" s="65"/>
-      <c r="L52" s="63"/>
-      <c r="M52" s="64"/>
-      <c r="N52" s="64"/>
-      <c r="O52" s="65"/>
+      <c r="B52" s="37"/>
+      <c r="C52" s="38"/>
+      <c r="D52" s="39"/>
+      <c r="E52" s="37"/>
+      <c r="F52" s="38"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="37"/>
+      <c r="I52" s="38"/>
+      <c r="J52" s="38"/>
+      <c r="K52" s="39"/>
+      <c r="L52" s="37"/>
+      <c r="M52" s="38"/>
+      <c r="N52" s="38"/>
+      <c r="O52" s="39"/>
     </row>
     <row r="53" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B53" s="48" t="s">
+      <c r="B53" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C53" s="28"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="48" t="s">
+      <c r="C53" s="26"/>
+      <c r="D53" s="27"/>
+      <c r="E53" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="F53" s="28"/>
-      <c r="G53" s="26"/>
-      <c r="H53" s="48" t="s">
+      <c r="F53" s="26"/>
+      <c r="G53" s="27"/>
+      <c r="H53" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="I53" s="28"/>
-      <c r="J53" s="28"/>
-      <c r="K53" s="26"/>
-      <c r="L53" s="48" t="s">
+      <c r="I53" s="26"/>
+      <c r="J53" s="26"/>
+      <c r="K53" s="27"/>
+      <c r="L53" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="M53" s="28"/>
-      <c r="N53" s="28"/>
-      <c r="O53" s="26"/>
+      <c r="M53" s="26"/>
+      <c r="N53" s="26"/>
+      <c r="O53" s="27"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B54" s="27" t="s">
+      <c r="B54" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="C54" s="61"/>
-      <c r="D54" s="62"/>
-      <c r="E54" s="27" t="s">
+      <c r="C54" s="35"/>
+      <c r="D54" s="36"/>
+      <c r="E54" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="F54" s="61"/>
-      <c r="G54" s="62"/>
-      <c r="H54" s="27"/>
-      <c r="I54" s="61"/>
-      <c r="J54" s="61"/>
-      <c r="K54" s="62"/>
-      <c r="L54" s="27"/>
-      <c r="M54" s="61"/>
-      <c r="N54" s="61"/>
-      <c r="O54" s="62"/>
+      <c r="F54" s="35"/>
+      <c r="G54" s="36"/>
+      <c r="H54" s="25"/>
+      <c r="I54" s="35"/>
+      <c r="J54" s="35"/>
+      <c r="K54" s="36"/>
+      <c r="L54" s="25"/>
+      <c r="M54" s="35"/>
+      <c r="N54" s="35"/>
+      <c r="O54" s="36"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B55" s="63"/>
-      <c r="C55" s="64"/>
-      <c r="D55" s="65"/>
-      <c r="E55" s="63"/>
-      <c r="F55" s="64"/>
-      <c r="G55" s="65"/>
-      <c r="H55" s="63"/>
-      <c r="I55" s="64"/>
-      <c r="J55" s="64"/>
-      <c r="K55" s="65"/>
-      <c r="L55" s="63"/>
-      <c r="M55" s="64"/>
-      <c r="N55" s="64"/>
-      <c r="O55" s="65"/>
+      <c r="B55" s="37"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="39"/>
+      <c r="E55" s="37"/>
+      <c r="F55" s="38"/>
+      <c r="G55" s="39"/>
+      <c r="H55" s="37"/>
+      <c r="I55" s="38"/>
+      <c r="J55" s="38"/>
+      <c r="K55" s="39"/>
+      <c r="L55" s="37"/>
+      <c r="M55" s="38"/>
+      <c r="N55" s="38"/>
+      <c r="O55" s="39"/>
     </row>
     <row r="56" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B56" s="48" t="s">
+      <c r="B56" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C56" s="28"/>
-      <c r="D56" s="26"/>
-      <c r="E56" s="48" t="s">
+      <c r="C56" s="26"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="F56" s="28"/>
-      <c r="G56" s="26"/>
-      <c r="H56" s="48" t="s">
+      <c r="F56" s="26"/>
+      <c r="G56" s="27"/>
+      <c r="H56" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="I56" s="28"/>
-      <c r="J56" s="28"/>
-      <c r="K56" s="26"/>
-      <c r="L56" s="48" t="s">
+      <c r="I56" s="26"/>
+      <c r="J56" s="26"/>
+      <c r="K56" s="27"/>
+      <c r="L56" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="M56" s="28"/>
-      <c r="N56" s="28"/>
-      <c r="O56" s="26"/>
+      <c r="M56" s="26"/>
+      <c r="N56" s="26"/>
+      <c r="O56" s="27"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B57" s="27" t="s">
+      <c r="B57" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="C57" s="61"/>
-      <c r="D57" s="62"/>
-      <c r="E57" s="27" t="s">
+      <c r="C57" s="35"/>
+      <c r="D57" s="36"/>
+      <c r="E57" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="F57" s="61"/>
-      <c r="G57" s="62"/>
-      <c r="H57" s="27"/>
-      <c r="I57" s="61"/>
-      <c r="J57" s="61"/>
-      <c r="K57" s="62"/>
-      <c r="L57" s="27"/>
-      <c r="M57" s="61"/>
-      <c r="N57" s="61"/>
-      <c r="O57" s="62"/>
+      <c r="F57" s="35"/>
+      <c r="G57" s="36"/>
+      <c r="H57" s="25"/>
+      <c r="I57" s="35"/>
+      <c r="J57" s="35"/>
+      <c r="K57" s="36"/>
+      <c r="L57" s="25"/>
+      <c r="M57" s="35"/>
+      <c r="N57" s="35"/>
+      <c r="O57" s="36"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B58" s="63"/>
-      <c r="C58" s="64"/>
-      <c r="D58" s="65"/>
-      <c r="E58" s="63"/>
-      <c r="F58" s="64"/>
-      <c r="G58" s="65"/>
-      <c r="H58" s="63"/>
-      <c r="I58" s="64"/>
-      <c r="J58" s="64"/>
-      <c r="K58" s="65"/>
-      <c r="L58" s="63"/>
-      <c r="M58" s="64"/>
-      <c r="N58" s="64"/>
-      <c r="O58" s="65"/>
+      <c r="B58" s="37"/>
+      <c r="C58" s="38"/>
+      <c r="D58" s="39"/>
+      <c r="E58" s="37"/>
+      <c r="F58" s="38"/>
+      <c r="G58" s="39"/>
+      <c r="H58" s="37"/>
+      <c r="I58" s="38"/>
+      <c r="J58" s="38"/>
+      <c r="K58" s="39"/>
+      <c r="L58" s="37"/>
+      <c r="M58" s="38"/>
+      <c r="N58" s="38"/>
+      <c r="O58" s="39"/>
     </row>
     <row r="59" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B59" s="5"/>
@@ -3062,41 +3062,41 @@
       <c r="O59" s="5"/>
     </row>
     <row r="60" spans="2:15" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B60" s="35" t="s">
+      <c r="B60" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="C60" s="36"/>
-      <c r="D60" s="36"/>
-      <c r="E60" s="36"/>
-      <c r="F60" s="36"/>
-      <c r="G60" s="36"/>
-      <c r="H60" s="36"/>
-      <c r="I60" s="36"/>
-      <c r="J60" s="36"/>
-      <c r="K60" s="36"/>
-      <c r="L60" s="36"/>
-      <c r="M60" s="36"/>
-      <c r="N60" s="36"/>
-      <c r="O60" s="37"/>
+      <c r="C60" s="43"/>
+      <c r="D60" s="43"/>
+      <c r="E60" s="43"/>
+      <c r="F60" s="43"/>
+      <c r="G60" s="43"/>
+      <c r="H60" s="43"/>
+      <c r="I60" s="43"/>
+      <c r="J60" s="43"/>
+      <c r="K60" s="43"/>
+      <c r="L60" s="43"/>
+      <c r="M60" s="43"/>
+      <c r="N60" s="43"/>
+      <c r="O60" s="44"/>
     </row>
     <row r="61" spans="2:15" ht="33" x14ac:dyDescent="0.3">
-      <c r="B61" s="80" t="s">
+      <c r="B61" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="C61" s="26"/>
+      <c r="C61" s="27"/>
       <c r="D61" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E61" s="80" t="s">
+      <c r="E61" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="F61" s="28"/>
-      <c r="G61" s="26"/>
-      <c r="H61" s="80" t="s">
+      <c r="F61" s="26"/>
+      <c r="G61" s="27"/>
+      <c r="H61" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="I61" s="28"/>
-      <c r="J61" s="26"/>
+      <c r="I61" s="26"/>
+      <c r="J61" s="27"/>
       <c r="K61" s="7" t="s">
         <v>44</v>
       </c>
@@ -3106,340 +3106,340 @@
       <c r="M61" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="N61" s="80" t="s">
+      <c r="N61" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="O61" s="26"/>
+      <c r="O61" s="27"/>
     </row>
     <row r="62" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B62" s="73" t="s">
+      <c r="B62" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="C62" s="62"/>
+      <c r="C62" s="36"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="27"/>
-      <c r="F62" s="28"/>
-      <c r="G62" s="26"/>
-      <c r="H62" s="27"/>
-      <c r="I62" s="28"/>
-      <c r="J62" s="26"/>
+      <c r="E62" s="25"/>
+      <c r="F62" s="26"/>
+      <c r="G62" s="27"/>
+      <c r="H62" s="25"/>
+      <c r="I62" s="26"/>
+      <c r="J62" s="27"/>
       <c r="K62" s="4"/>
       <c r="L62" s="4"/>
       <c r="M62" s="4"/>
-      <c r="N62" s="27"/>
-      <c r="O62" s="26"/>
+      <c r="N62" s="25"/>
+      <c r="O62" s="27"/>
     </row>
     <row r="63" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B63" s="70"/>
-      <c r="C63" s="72"/>
+      <c r="B63" s="47"/>
+      <c r="C63" s="48"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="27"/>
-      <c r="F63" s="28"/>
-      <c r="G63" s="26"/>
-      <c r="H63" s="27"/>
-      <c r="I63" s="28"/>
-      <c r="J63" s="26"/>
+      <c r="E63" s="25"/>
+      <c r="F63" s="26"/>
+      <c r="G63" s="27"/>
+      <c r="H63" s="25"/>
+      <c r="I63" s="26"/>
+      <c r="J63" s="27"/>
       <c r="K63" s="4"/>
       <c r="L63" s="4"/>
       <c r="M63" s="4"/>
-      <c r="N63" s="27"/>
-      <c r="O63" s="26"/>
+      <c r="N63" s="25"/>
+      <c r="O63" s="27"/>
     </row>
     <row r="64" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B64" s="70"/>
-      <c r="C64" s="72"/>
+      <c r="B64" s="47"/>
+      <c r="C64" s="48"/>
       <c r="D64" s="4"/>
-      <c r="E64" s="27"/>
-      <c r="F64" s="28"/>
-      <c r="G64" s="26"/>
-      <c r="H64" s="27"/>
-      <c r="I64" s="28"/>
-      <c r="J64" s="26"/>
+      <c r="E64" s="25"/>
+      <c r="F64" s="26"/>
+      <c r="G64" s="27"/>
+      <c r="H64" s="25"/>
+      <c r="I64" s="26"/>
+      <c r="J64" s="27"/>
       <c r="K64" s="4"/>
       <c r="L64" s="4"/>
       <c r="M64" s="4"/>
-      <c r="N64" s="27"/>
-      <c r="O64" s="26"/>
+      <c r="N64" s="25"/>
+      <c r="O64" s="27"/>
     </row>
     <row r="65" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B65" s="63"/>
-      <c r="C65" s="65"/>
+      <c r="B65" s="37"/>
+      <c r="C65" s="39"/>
       <c r="D65" s="4"/>
-      <c r="E65" s="27"/>
-      <c r="F65" s="28"/>
-      <c r="G65" s="26"/>
-      <c r="H65" s="27"/>
-      <c r="I65" s="28"/>
-      <c r="J65" s="26"/>
+      <c r="E65" s="25"/>
+      <c r="F65" s="26"/>
+      <c r="G65" s="27"/>
+      <c r="H65" s="25"/>
+      <c r="I65" s="26"/>
+      <c r="J65" s="27"/>
       <c r="K65" s="4"/>
       <c r="L65" s="4"/>
       <c r="M65" s="4"/>
-      <c r="N65" s="27"/>
-      <c r="O65" s="26"/>
+      <c r="N65" s="25"/>
+      <c r="O65" s="27"/>
     </row>
     <row r="66" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B66" s="73" t="s">
+      <c r="B66" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="C66" s="62"/>
+      <c r="C66" s="36"/>
       <c r="D66" s="4"/>
-      <c r="E66" s="27"/>
-      <c r="F66" s="28"/>
-      <c r="G66" s="26"/>
-      <c r="H66" s="27"/>
-      <c r="I66" s="28"/>
-      <c r="J66" s="26"/>
+      <c r="E66" s="25"/>
+      <c r="F66" s="26"/>
+      <c r="G66" s="27"/>
+      <c r="H66" s="25"/>
+      <c r="I66" s="26"/>
+      <c r="J66" s="27"/>
       <c r="K66" s="4"/>
       <c r="L66" s="4"/>
       <c r="M66" s="4"/>
-      <c r="N66" s="27"/>
-      <c r="O66" s="26"/>
+      <c r="N66" s="25"/>
+      <c r="O66" s="27"/>
     </row>
     <row r="67" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B67" s="70"/>
-      <c r="C67" s="72"/>
+      <c r="B67" s="47"/>
+      <c r="C67" s="48"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="27"/>
-      <c r="F67" s="28"/>
-      <c r="G67" s="26"/>
-      <c r="H67" s="27"/>
-      <c r="I67" s="28"/>
-      <c r="J67" s="26"/>
+      <c r="E67" s="25"/>
+      <c r="F67" s="26"/>
+      <c r="G67" s="27"/>
+      <c r="H67" s="25"/>
+      <c r="I67" s="26"/>
+      <c r="J67" s="27"/>
       <c r="K67" s="4"/>
       <c r="L67" s="4"/>
       <c r="M67" s="4"/>
-      <c r="N67" s="27"/>
-      <c r="O67" s="26"/>
+      <c r="N67" s="25"/>
+      <c r="O67" s="27"/>
     </row>
     <row r="68" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B68" s="70"/>
-      <c r="C68" s="72"/>
+      <c r="B68" s="47"/>
+      <c r="C68" s="48"/>
       <c r="D68" s="4"/>
-      <c r="E68" s="27"/>
-      <c r="F68" s="28"/>
-      <c r="G68" s="26"/>
-      <c r="H68" s="27"/>
-      <c r="I68" s="28"/>
-      <c r="J68" s="26"/>
+      <c r="E68" s="25"/>
+      <c r="F68" s="26"/>
+      <c r="G68" s="27"/>
+      <c r="H68" s="25"/>
+      <c r="I68" s="26"/>
+      <c r="J68" s="27"/>
       <c r="K68" s="4"/>
       <c r="L68" s="4"/>
       <c r="M68" s="4"/>
-      <c r="N68" s="27"/>
-      <c r="O68" s="26"/>
+      <c r="N68" s="25"/>
+      <c r="O68" s="27"/>
     </row>
     <row r="69" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B69" s="63"/>
-      <c r="C69" s="65"/>
+      <c r="B69" s="37"/>
+      <c r="C69" s="39"/>
       <c r="D69" s="4"/>
-      <c r="E69" s="27"/>
-      <c r="F69" s="28"/>
-      <c r="G69" s="26"/>
-      <c r="H69" s="27"/>
-      <c r="I69" s="28"/>
-      <c r="J69" s="26"/>
+      <c r="E69" s="25"/>
+      <c r="F69" s="26"/>
+      <c r="G69" s="27"/>
+      <c r="H69" s="25"/>
+      <c r="I69" s="26"/>
+      <c r="J69" s="27"/>
       <c r="K69" s="4"/>
       <c r="L69" s="4"/>
       <c r="M69" s="4"/>
-      <c r="N69" s="27"/>
-      <c r="O69" s="26"/>
+      <c r="N69" s="25"/>
+      <c r="O69" s="27"/>
     </row>
     <row r="70" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B70" s="73" t="s">
+      <c r="B70" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="C70" s="62"/>
+      <c r="C70" s="36"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="27"/>
-      <c r="F70" s="28"/>
-      <c r="G70" s="26"/>
-      <c r="H70" s="27"/>
-      <c r="I70" s="28"/>
-      <c r="J70" s="26"/>
+      <c r="E70" s="25"/>
+      <c r="F70" s="26"/>
+      <c r="G70" s="27"/>
+      <c r="H70" s="25"/>
+      <c r="I70" s="26"/>
+      <c r="J70" s="27"/>
       <c r="K70" s="4"/>
       <c r="L70" s="4"/>
       <c r="M70" s="4"/>
-      <c r="N70" s="27"/>
-      <c r="O70" s="26"/>
+      <c r="N70" s="25"/>
+      <c r="O70" s="27"/>
     </row>
     <row r="71" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B71" s="70"/>
-      <c r="C71" s="72"/>
+      <c r="B71" s="47"/>
+      <c r="C71" s="48"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="27"/>
-      <c r="F71" s="28"/>
-      <c r="G71" s="26"/>
-      <c r="H71" s="27"/>
-      <c r="I71" s="28"/>
-      <c r="J71" s="26"/>
+      <c r="E71" s="25"/>
+      <c r="F71" s="26"/>
+      <c r="G71" s="27"/>
+      <c r="H71" s="25"/>
+      <c r="I71" s="26"/>
+      <c r="J71" s="27"/>
       <c r="K71" s="4"/>
       <c r="L71" s="4"/>
       <c r="M71" s="4"/>
-      <c r="N71" s="27"/>
-      <c r="O71" s="26"/>
+      <c r="N71" s="25"/>
+      <c r="O71" s="27"/>
     </row>
     <row r="72" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B72" s="70"/>
-      <c r="C72" s="72"/>
+      <c r="B72" s="47"/>
+      <c r="C72" s="48"/>
       <c r="D72" s="4"/>
-      <c r="E72" s="27"/>
-      <c r="F72" s="28"/>
-      <c r="G72" s="26"/>
-      <c r="H72" s="27"/>
-      <c r="I72" s="28"/>
-      <c r="J72" s="26"/>
+      <c r="E72" s="25"/>
+      <c r="F72" s="26"/>
+      <c r="G72" s="27"/>
+      <c r="H72" s="25"/>
+      <c r="I72" s="26"/>
+      <c r="J72" s="27"/>
       <c r="K72" s="4"/>
       <c r="L72" s="4"/>
       <c r="M72" s="4"/>
-      <c r="N72" s="27"/>
-      <c r="O72" s="26"/>
+      <c r="N72" s="25"/>
+      <c r="O72" s="27"/>
     </row>
     <row r="73" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B73" s="63"/>
-      <c r="C73" s="65"/>
+      <c r="B73" s="37"/>
+      <c r="C73" s="39"/>
       <c r="D73" s="4"/>
-      <c r="E73" s="27"/>
-      <c r="F73" s="28"/>
-      <c r="G73" s="26"/>
-      <c r="H73" s="27"/>
-      <c r="I73" s="28"/>
-      <c r="J73" s="26"/>
+      <c r="E73" s="25"/>
+      <c r="F73" s="26"/>
+      <c r="G73" s="27"/>
+      <c r="H73" s="25"/>
+      <c r="I73" s="26"/>
+      <c r="J73" s="27"/>
       <c r="K73" s="4"/>
       <c r="L73" s="4"/>
       <c r="M73" s="4"/>
-      <c r="N73" s="27"/>
-      <c r="O73" s="26"/>
+      <c r="N73" s="25"/>
+      <c r="O73" s="27"/>
     </row>
     <row r="74" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B74" s="73" t="s">
+      <c r="B74" s="46" t="s">
         <v>127</v>
       </c>
-      <c r="C74" s="62"/>
+      <c r="C74" s="36"/>
       <c r="D74" s="4"/>
-      <c r="E74" s="27"/>
-      <c r="F74" s="28"/>
-      <c r="G74" s="26"/>
-      <c r="H74" s="27"/>
-      <c r="I74" s="28"/>
-      <c r="J74" s="26"/>
+      <c r="E74" s="25"/>
+      <c r="F74" s="26"/>
+      <c r="G74" s="27"/>
+      <c r="H74" s="25"/>
+      <c r="I74" s="26"/>
+      <c r="J74" s="27"/>
       <c r="K74" s="4"/>
       <c r="L74" s="4"/>
       <c r="M74" s="4"/>
-      <c r="N74" s="27"/>
-      <c r="O74" s="26"/>
+      <c r="N74" s="25"/>
+      <c r="O74" s="27"/>
     </row>
     <row r="75" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B75" s="70"/>
-      <c r="C75" s="72"/>
+      <c r="B75" s="47"/>
+      <c r="C75" s="48"/>
       <c r="D75" s="4"/>
-      <c r="E75" s="27"/>
-      <c r="F75" s="28"/>
-      <c r="G75" s="26"/>
-      <c r="H75" s="27"/>
-      <c r="I75" s="28"/>
-      <c r="J75" s="26"/>
+      <c r="E75" s="25"/>
+      <c r="F75" s="26"/>
+      <c r="G75" s="27"/>
+      <c r="H75" s="25"/>
+      <c r="I75" s="26"/>
+      <c r="J75" s="27"/>
       <c r="K75" s="4"/>
       <c r="L75" s="4"/>
       <c r="M75" s="4"/>
-      <c r="N75" s="27"/>
-      <c r="O75" s="26"/>
+      <c r="N75" s="25"/>
+      <c r="O75" s="27"/>
     </row>
     <row r="76" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B76" s="70"/>
-      <c r="C76" s="72"/>
+      <c r="B76" s="47"/>
+      <c r="C76" s="48"/>
       <c r="D76" s="4"/>
-      <c r="E76" s="27"/>
-      <c r="F76" s="28"/>
-      <c r="G76" s="26"/>
-      <c r="H76" s="27"/>
-      <c r="I76" s="28"/>
-      <c r="J76" s="26"/>
+      <c r="E76" s="25"/>
+      <c r="F76" s="26"/>
+      <c r="G76" s="27"/>
+      <c r="H76" s="25"/>
+      <c r="I76" s="26"/>
+      <c r="J76" s="27"/>
       <c r="K76" s="4"/>
       <c r="L76" s="4"/>
       <c r="M76" s="4"/>
-      <c r="N76" s="27"/>
-      <c r="O76" s="26"/>
+      <c r="N76" s="25"/>
+      <c r="O76" s="27"/>
     </row>
     <row r="77" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B77" s="63"/>
-      <c r="C77" s="65"/>
+      <c r="B77" s="37"/>
+      <c r="C77" s="39"/>
       <c r="D77" s="4"/>
-      <c r="E77" s="27"/>
-      <c r="F77" s="28"/>
-      <c r="G77" s="26"/>
-      <c r="H77" s="27"/>
-      <c r="I77" s="28"/>
-      <c r="J77" s="26"/>
+      <c r="E77" s="25"/>
+      <c r="F77" s="26"/>
+      <c r="G77" s="27"/>
+      <c r="H77" s="25"/>
+      <c r="I77" s="26"/>
+      <c r="J77" s="27"/>
       <c r="K77" s="4"/>
       <c r="L77" s="4"/>
       <c r="M77" s="4"/>
-      <c r="N77" s="27"/>
-      <c r="O77" s="26"/>
+      <c r="N77" s="25"/>
+      <c r="O77" s="27"/>
     </row>
     <row r="78" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B78" s="73" t="s">
+      <c r="B78" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="C78" s="62"/>
+      <c r="C78" s="36"/>
       <c r="D78" s="4"/>
-      <c r="E78" s="27"/>
-      <c r="F78" s="28"/>
-      <c r="G78" s="26"/>
-      <c r="H78" s="27"/>
-      <c r="I78" s="28"/>
-      <c r="J78" s="26"/>
+      <c r="E78" s="25"/>
+      <c r="F78" s="26"/>
+      <c r="G78" s="27"/>
+      <c r="H78" s="25"/>
+      <c r="I78" s="26"/>
+      <c r="J78" s="27"/>
       <c r="K78" s="4"/>
       <c r="L78" s="4"/>
       <c r="M78" s="4"/>
-      <c r="N78" s="27"/>
-      <c r="O78" s="26"/>
+      <c r="N78" s="25"/>
+      <c r="O78" s="27"/>
     </row>
     <row r="79" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B79" s="70"/>
-      <c r="C79" s="72"/>
+      <c r="B79" s="47"/>
+      <c r="C79" s="48"/>
       <c r="D79" s="4"/>
-      <c r="E79" s="27"/>
-      <c r="F79" s="28"/>
-      <c r="G79" s="26"/>
-      <c r="H79" s="27"/>
-      <c r="I79" s="28"/>
-      <c r="J79" s="26"/>
+      <c r="E79" s="25"/>
+      <c r="F79" s="26"/>
+      <c r="G79" s="27"/>
+      <c r="H79" s="25"/>
+      <c r="I79" s="26"/>
+      <c r="J79" s="27"/>
       <c r="K79" s="4"/>
       <c r="L79" s="4"/>
       <c r="M79" s="4"/>
-      <c r="N79" s="27"/>
-      <c r="O79" s="26"/>
+      <c r="N79" s="25"/>
+      <c r="O79" s="27"/>
     </row>
     <row r="80" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B80" s="70"/>
-      <c r="C80" s="72"/>
+      <c r="B80" s="47"/>
+      <c r="C80" s="48"/>
       <c r="D80" s="4"/>
-      <c r="E80" s="27"/>
-      <c r="F80" s="28"/>
-      <c r="G80" s="26"/>
-      <c r="H80" s="27"/>
-      <c r="I80" s="28"/>
-      <c r="J80" s="26"/>
+      <c r="E80" s="25"/>
+      <c r="F80" s="26"/>
+      <c r="G80" s="27"/>
+      <c r="H80" s="25"/>
+      <c r="I80" s="26"/>
+      <c r="J80" s="27"/>
       <c r="K80" s="4"/>
       <c r="L80" s="4"/>
       <c r="M80" s="4"/>
-      <c r="N80" s="27"/>
-      <c r="O80" s="26"/>
+      <c r="N80" s="25"/>
+      <c r="O80" s="27"/>
     </row>
     <row r="81" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B81" s="63"/>
-      <c r="C81" s="65"/>
+      <c r="B81" s="37"/>
+      <c r="C81" s="39"/>
       <c r="D81" s="4"/>
-      <c r="E81" s="27"/>
-      <c r="F81" s="28"/>
-      <c r="G81" s="26"/>
-      <c r="H81" s="27"/>
-      <c r="I81" s="28"/>
-      <c r="J81" s="26"/>
+      <c r="E81" s="25"/>
+      <c r="F81" s="26"/>
+      <c r="G81" s="27"/>
+      <c r="H81" s="25"/>
+      <c r="I81" s="26"/>
+      <c r="J81" s="27"/>
       <c r="K81" s="4"/>
       <c r="L81" s="4"/>
       <c r="M81" s="4"/>
-      <c r="N81" s="27"/>
-      <c r="O81" s="26"/>
+      <c r="N81" s="25"/>
+      <c r="O81" s="27"/>
     </row>
     <row r="82" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B82" s="5"/>
@@ -3458,118 +3458,118 @@
       <c r="O82" s="5"/>
     </row>
     <row r="83" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B83" s="35" t="s">
+      <c r="B83" s="42" t="s">
         <v>163</v>
       </c>
-      <c r="C83" s="36"/>
-      <c r="D83" s="36"/>
-      <c r="E83" s="36"/>
-      <c r="F83" s="36"/>
-      <c r="G83" s="36"/>
-      <c r="H83" s="36"/>
-      <c r="I83" s="36"/>
-      <c r="J83" s="36"/>
-      <c r="K83" s="36"/>
-      <c r="L83" s="36"/>
-      <c r="M83" s="36"/>
-      <c r="N83" s="36"/>
-      <c r="O83" s="37"/>
+      <c r="C83" s="43"/>
+      <c r="D83" s="43"/>
+      <c r="E83" s="43"/>
+      <c r="F83" s="43"/>
+      <c r="G83" s="43"/>
+      <c r="H83" s="43"/>
+      <c r="I83" s="43"/>
+      <c r="J83" s="43"/>
+      <c r="K83" s="43"/>
+      <c r="L83" s="43"/>
+      <c r="M83" s="43"/>
+      <c r="N83" s="43"/>
+      <c r="O83" s="44"/>
     </row>
     <row r="84" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B84" s="38" t="s">
+      <c r="B84" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C84" s="26"/>
-      <c r="D84" s="38" t="s">
+      <c r="C84" s="27"/>
+      <c r="D84" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="E84" s="28"/>
-      <c r="F84" s="28"/>
-      <c r="G84" s="28"/>
-      <c r="H84" s="28"/>
-      <c r="I84" s="26"/>
-      <c r="J84" s="38" t="s">
+      <c r="E84" s="26"/>
+      <c r="F84" s="26"/>
+      <c r="G84" s="26"/>
+      <c r="H84" s="26"/>
+      <c r="I84" s="27"/>
+      <c r="J84" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="K84" s="28"/>
-      <c r="L84" s="26"/>
-      <c r="M84" s="38" t="s">
+      <c r="K84" s="26"/>
+      <c r="L84" s="27"/>
+      <c r="M84" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="N84" s="28"/>
-      <c r="O84" s="26"/>
+      <c r="N84" s="26"/>
+      <c r="O84" s="27"/>
     </row>
     <row r="85" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B85" s="25" t="s">
+      <c r="B85" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="C85" s="26"/>
-      <c r="D85" s="27"/>
-      <c r="E85" s="28"/>
-      <c r="F85" s="28"/>
-      <c r="G85" s="28"/>
-      <c r="H85" s="28"/>
-      <c r="I85" s="26"/>
-      <c r="J85" s="27"/>
-      <c r="K85" s="28"/>
-      <c r="L85" s="26"/>
-      <c r="M85" s="27"/>
-      <c r="N85" s="28"/>
-      <c r="O85" s="26"/>
+      <c r="C85" s="27"/>
+      <c r="D85" s="25"/>
+      <c r="E85" s="26"/>
+      <c r="F85" s="26"/>
+      <c r="G85" s="26"/>
+      <c r="H85" s="26"/>
+      <c r="I85" s="27"/>
+      <c r="J85" s="25"/>
+      <c r="K85" s="26"/>
+      <c r="L85" s="27"/>
+      <c r="M85" s="25"/>
+      <c r="N85" s="26"/>
+      <c r="O85" s="27"/>
     </row>
     <row r="86" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B86" s="25" t="s">
+      <c r="B86" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C86" s="26"/>
-      <c r="D86" s="27"/>
-      <c r="E86" s="28"/>
-      <c r="F86" s="28"/>
-      <c r="G86" s="28"/>
-      <c r="H86" s="28"/>
-      <c r="I86" s="26"/>
-      <c r="J86" s="27"/>
-      <c r="K86" s="28"/>
-      <c r="L86" s="26"/>
-      <c r="M86" s="27"/>
-      <c r="N86" s="28"/>
-      <c r="O86" s="26"/>
+      <c r="C86" s="27"/>
+      <c r="D86" s="25"/>
+      <c r="E86" s="26"/>
+      <c r="F86" s="26"/>
+      <c r="G86" s="26"/>
+      <c r="H86" s="26"/>
+      <c r="I86" s="27"/>
+      <c r="J86" s="25"/>
+      <c r="K86" s="26"/>
+      <c r="L86" s="27"/>
+      <c r="M86" s="25"/>
+      <c r="N86" s="26"/>
+      <c r="O86" s="27"/>
     </row>
     <row r="87" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B87" s="25" t="s">
+      <c r="B87" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="C87" s="26"/>
-      <c r="D87" s="27"/>
-      <c r="E87" s="28"/>
-      <c r="F87" s="28"/>
-      <c r="G87" s="28"/>
-      <c r="H87" s="28"/>
-      <c r="I87" s="26"/>
-      <c r="J87" s="27"/>
-      <c r="K87" s="28"/>
-      <c r="L87" s="26"/>
-      <c r="M87" s="27"/>
-      <c r="N87" s="28"/>
-      <c r="O87" s="26"/>
+      <c r="C87" s="27"/>
+      <c r="D87" s="25"/>
+      <c r="E87" s="26"/>
+      <c r="F87" s="26"/>
+      <c r="G87" s="26"/>
+      <c r="H87" s="26"/>
+      <c r="I87" s="27"/>
+      <c r="J87" s="25"/>
+      <c r="K87" s="26"/>
+      <c r="L87" s="27"/>
+      <c r="M87" s="25"/>
+      <c r="N87" s="26"/>
+      <c r="O87" s="27"/>
     </row>
     <row r="88" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B88" s="25" t="s">
+      <c r="B88" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="C88" s="26"/>
-      <c r="D88" s="27"/>
-      <c r="E88" s="28"/>
-      <c r="F88" s="28"/>
-      <c r="G88" s="28"/>
-      <c r="H88" s="28"/>
-      <c r="I88" s="26"/>
-      <c r="J88" s="27"/>
-      <c r="K88" s="28"/>
-      <c r="L88" s="26"/>
-      <c r="M88" s="27"/>
-      <c r="N88" s="28"/>
-      <c r="O88" s="26"/>
+      <c r="C88" s="27"/>
+      <c r="D88" s="25"/>
+      <c r="E88" s="26"/>
+      <c r="F88" s="26"/>
+      <c r="G88" s="26"/>
+      <c r="H88" s="26"/>
+      <c r="I88" s="27"/>
+      <c r="J88" s="25"/>
+      <c r="K88" s="26"/>
+      <c r="L88" s="27"/>
+      <c r="M88" s="25"/>
+      <c r="N88" s="26"/>
+      <c r="O88" s="27"/>
     </row>
     <row r="89" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B89" s="5"/>
@@ -3588,154 +3588,154 @@
       <c r="O89" s="5"/>
     </row>
     <row r="90" spans="2:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="35" t="s">
+      <c r="B90" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="C90" s="36"/>
-      <c r="D90" s="36"/>
-      <c r="E90" s="36"/>
-      <c r="F90" s="36"/>
-      <c r="G90" s="36"/>
-      <c r="H90" s="36"/>
-      <c r="I90" s="36"/>
-      <c r="J90" s="36"/>
-      <c r="K90" s="36"/>
-      <c r="L90" s="36"/>
-      <c r="M90" s="36"/>
-      <c r="N90" s="36"/>
-      <c r="O90" s="37"/>
+      <c r="C90" s="43"/>
+      <c r="D90" s="43"/>
+      <c r="E90" s="43"/>
+      <c r="F90" s="43"/>
+      <c r="G90" s="43"/>
+      <c r="H90" s="43"/>
+      <c r="I90" s="43"/>
+      <c r="J90" s="43"/>
+      <c r="K90" s="43"/>
+      <c r="L90" s="43"/>
+      <c r="M90" s="43"/>
+      <c r="N90" s="43"/>
+      <c r="O90" s="44"/>
     </row>
     <row r="91" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B91" s="38" t="s">
+      <c r="B91" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="C91" s="28"/>
-      <c r="D91" s="28"/>
-      <c r="E91" s="26"/>
-      <c r="F91" s="38" t="s">
+      <c r="C91" s="26"/>
+      <c r="D91" s="26"/>
+      <c r="E91" s="27"/>
+      <c r="F91" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="G91" s="26"/>
-      <c r="H91" s="38" t="s">
+      <c r="G91" s="27"/>
+      <c r="H91" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="I91" s="28"/>
-      <c r="J91" s="28"/>
-      <c r="K91" s="28"/>
-      <c r="L91" s="28"/>
-      <c r="M91" s="26"/>
-      <c r="N91" s="38" t="s">
+      <c r="I91" s="26"/>
+      <c r="J91" s="26"/>
+      <c r="K91" s="26"/>
+      <c r="L91" s="26"/>
+      <c r="M91" s="27"/>
+      <c r="N91" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="O91" s="26"/>
+      <c r="O91" s="27"/>
     </row>
     <row r="92" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B92" s="25" t="s">
+      <c r="B92" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="C92" s="28"/>
-      <c r="D92" s="28"/>
-      <c r="E92" s="26"/>
-      <c r="F92" s="27"/>
-      <c r="G92" s="26"/>
-      <c r="H92" s="27"/>
-      <c r="I92" s="28"/>
-      <c r="J92" s="28"/>
-      <c r="K92" s="28"/>
-      <c r="L92" s="28"/>
-      <c r="M92" s="26"/>
-      <c r="N92" s="27"/>
-      <c r="O92" s="26"/>
+      <c r="C92" s="26"/>
+      <c r="D92" s="26"/>
+      <c r="E92" s="27"/>
+      <c r="F92" s="25"/>
+      <c r="G92" s="27"/>
+      <c r="H92" s="25"/>
+      <c r="I92" s="26"/>
+      <c r="J92" s="26"/>
+      <c r="K92" s="26"/>
+      <c r="L92" s="26"/>
+      <c r="M92" s="27"/>
+      <c r="N92" s="25"/>
+      <c r="O92" s="27"/>
     </row>
     <row r="93" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B93" s="25" t="s">
+      <c r="B93" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C93" s="28"/>
-      <c r="D93" s="28"/>
-      <c r="E93" s="26"/>
-      <c r="F93" s="27"/>
-      <c r="G93" s="26"/>
-      <c r="H93" s="27"/>
-      <c r="I93" s="28"/>
-      <c r="J93" s="28"/>
-      <c r="K93" s="28"/>
-      <c r="L93" s="28"/>
-      <c r="M93" s="26"/>
-      <c r="N93" s="27"/>
-      <c r="O93" s="26"/>
+      <c r="C93" s="26"/>
+      <c r="D93" s="26"/>
+      <c r="E93" s="27"/>
+      <c r="F93" s="25"/>
+      <c r="G93" s="27"/>
+      <c r="H93" s="25"/>
+      <c r="I93" s="26"/>
+      <c r="J93" s="26"/>
+      <c r="K93" s="26"/>
+      <c r="L93" s="26"/>
+      <c r="M93" s="27"/>
+      <c r="N93" s="25"/>
+      <c r="O93" s="27"/>
     </row>
     <row r="94" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B94" s="25" t="s">
+      <c r="B94" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="C94" s="28"/>
-      <c r="D94" s="28"/>
-      <c r="E94" s="26"/>
-      <c r="F94" s="27"/>
-      <c r="G94" s="26"/>
-      <c r="H94" s="27"/>
-      <c r="I94" s="28"/>
-      <c r="J94" s="28"/>
-      <c r="K94" s="28"/>
-      <c r="L94" s="28"/>
-      <c r="M94" s="26"/>
-      <c r="N94" s="27"/>
-      <c r="O94" s="26"/>
+      <c r="C94" s="26"/>
+      <c r="D94" s="26"/>
+      <c r="E94" s="27"/>
+      <c r="F94" s="25"/>
+      <c r="G94" s="27"/>
+      <c r="H94" s="25"/>
+      <c r="I94" s="26"/>
+      <c r="J94" s="26"/>
+      <c r="K94" s="26"/>
+      <c r="L94" s="26"/>
+      <c r="M94" s="27"/>
+      <c r="N94" s="25"/>
+      <c r="O94" s="27"/>
     </row>
     <row r="95" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B95" s="25" t="s">
+      <c r="B95" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="C95" s="28"/>
-      <c r="D95" s="28"/>
-      <c r="E95" s="26"/>
-      <c r="F95" s="27"/>
-      <c r="G95" s="26"/>
-      <c r="H95" s="27"/>
-      <c r="I95" s="28"/>
-      <c r="J95" s="28"/>
-      <c r="K95" s="28"/>
-      <c r="L95" s="28"/>
-      <c r="M95" s="26"/>
-      <c r="N95" s="27"/>
-      <c r="O95" s="26"/>
+      <c r="C95" s="26"/>
+      <c r="D95" s="26"/>
+      <c r="E95" s="27"/>
+      <c r="F95" s="25"/>
+      <c r="G95" s="27"/>
+      <c r="H95" s="25"/>
+      <c r="I95" s="26"/>
+      <c r="J95" s="26"/>
+      <c r="K95" s="26"/>
+      <c r="L95" s="26"/>
+      <c r="M95" s="27"/>
+      <c r="N95" s="25"/>
+      <c r="O95" s="27"/>
     </row>
     <row r="96" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B96" s="25" t="s">
+      <c r="B96" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="C96" s="28"/>
-      <c r="D96" s="28"/>
-      <c r="E96" s="26"/>
-      <c r="F96" s="27"/>
-      <c r="G96" s="26"/>
-      <c r="H96" s="27"/>
-      <c r="I96" s="28"/>
-      <c r="J96" s="28"/>
-      <c r="K96" s="28"/>
-      <c r="L96" s="28"/>
-      <c r="M96" s="26"/>
-      <c r="N96" s="27"/>
-      <c r="O96" s="26"/>
+      <c r="C96" s="26"/>
+      <c r="D96" s="26"/>
+      <c r="E96" s="27"/>
+      <c r="F96" s="25"/>
+      <c r="G96" s="27"/>
+      <c r="H96" s="25"/>
+      <c r="I96" s="26"/>
+      <c r="J96" s="26"/>
+      <c r="K96" s="26"/>
+      <c r="L96" s="26"/>
+      <c r="M96" s="27"/>
+      <c r="N96" s="25"/>
+      <c r="O96" s="27"/>
     </row>
     <row r="97" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B97" s="25" t="s">
+      <c r="B97" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="C97" s="28"/>
-      <c r="D97" s="28"/>
-      <c r="E97" s="26"/>
-      <c r="F97" s="27"/>
-      <c r="G97" s="26"/>
-      <c r="H97" s="27"/>
-      <c r="I97" s="28"/>
-      <c r="J97" s="28"/>
-      <c r="K97" s="28"/>
-      <c r="L97" s="28"/>
-      <c r="M97" s="26"/>
-      <c r="N97" s="27"/>
-      <c r="O97" s="26"/>
+      <c r="C97" s="26"/>
+      <c r="D97" s="26"/>
+      <c r="E97" s="27"/>
+      <c r="F97" s="25"/>
+      <c r="G97" s="27"/>
+      <c r="H97" s="25"/>
+      <c r="I97" s="26"/>
+      <c r="J97" s="26"/>
+      <c r="K97" s="26"/>
+      <c r="L97" s="26"/>
+      <c r="M97" s="27"/>
+      <c r="N97" s="25"/>
+      <c r="O97" s="27"/>
     </row>
     <row r="98" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B98" s="5"/>
@@ -3754,145 +3754,145 @@
       <c r="O98" s="5"/>
     </row>
     <row r="99" spans="2:15" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B99" s="35" t="s">
+      <c r="B99" s="42" t="s">
         <v>164</v>
       </c>
-      <c r="C99" s="36"/>
-      <c r="D99" s="36"/>
-      <c r="E99" s="36"/>
-      <c r="F99" s="36"/>
-      <c r="G99" s="36"/>
-      <c r="H99" s="36"/>
-      <c r="I99" s="36"/>
-      <c r="J99" s="36"/>
-      <c r="K99" s="36"/>
-      <c r="L99" s="36"/>
-      <c r="M99" s="36"/>
-      <c r="N99" s="36"/>
-      <c r="O99" s="37"/>
+      <c r="C99" s="43"/>
+      <c r="D99" s="43"/>
+      <c r="E99" s="43"/>
+      <c r="F99" s="43"/>
+      <c r="G99" s="43"/>
+      <c r="H99" s="43"/>
+      <c r="I99" s="43"/>
+      <c r="J99" s="43"/>
+      <c r="K99" s="43"/>
+      <c r="L99" s="43"/>
+      <c r="M99" s="43"/>
+      <c r="N99" s="43"/>
+      <c r="O99" s="44"/>
     </row>
     <row r="100" spans="2:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="18" t="s">
+      <c r="B100" s="89" t="s">
         <v>169</v>
       </c>
-      <c r="C100" s="19"/>
-      <c r="D100" s="19"/>
-      <c r="E100" s="19"/>
-      <c r="F100" s="19"/>
-      <c r="G100" s="19"/>
-      <c r="H100" s="19"/>
-      <c r="I100" s="19"/>
-      <c r="J100" s="19"/>
-      <c r="K100" s="19"/>
-      <c r="L100" s="19"/>
-      <c r="M100" s="19"/>
-      <c r="N100" s="19"/>
-      <c r="O100" s="19"/>
+      <c r="C100" s="90"/>
+      <c r="D100" s="90"/>
+      <c r="E100" s="90"/>
+      <c r="F100" s="90"/>
+      <c r="G100" s="90"/>
+      <c r="H100" s="90"/>
+      <c r="I100" s="90"/>
+      <c r="J100" s="90"/>
+      <c r="K100" s="90"/>
+      <c r="L100" s="90"/>
+      <c r="M100" s="90"/>
+      <c r="N100" s="90"/>
+      <c r="O100" s="90"/>
     </row>
     <row r="101" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B101" s="38" t="s">
+      <c r="B101" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C101" s="28"/>
-      <c r="D101" s="28"/>
-      <c r="E101" s="28"/>
-      <c r="F101" s="26"/>
-      <c r="G101" s="38" t="s">
+      <c r="C101" s="26"/>
+      <c r="D101" s="26"/>
+      <c r="E101" s="26"/>
+      <c r="F101" s="27"/>
+      <c r="G101" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="H101" s="28"/>
-      <c r="I101" s="26"/>
-      <c r="J101" s="20" t="s">
+      <c r="H101" s="26"/>
+      <c r="I101" s="27"/>
+      <c r="J101" s="31" t="s">
         <v>167</v>
       </c>
-      <c r="K101" s="86"/>
-      <c r="L101" s="21"/>
-      <c r="M101" s="20" t="s">
+      <c r="K101" s="32"/>
+      <c r="L101" s="33"/>
+      <c r="M101" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="N101" s="21"/>
+      <c r="N101" s="33"/>
       <c r="O101" s="7" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="102" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B102" s="27"/>
-      <c r="C102" s="28"/>
-      <c r="D102" s="28"/>
-      <c r="E102" s="28"/>
-      <c r="F102" s="26"/>
-      <c r="G102" s="27"/>
-      <c r="H102" s="28"/>
-      <c r="I102" s="26"/>
-      <c r="J102" s="22"/>
-      <c r="K102" s="23"/>
-      <c r="L102" s="23"/>
-      <c r="M102" s="22"/>
-      <c r="N102" s="24"/>
+      <c r="B102" s="25"/>
+      <c r="C102" s="26"/>
+      <c r="D102" s="26"/>
+      <c r="E102" s="26"/>
+      <c r="F102" s="27"/>
+      <c r="G102" s="25"/>
+      <c r="H102" s="26"/>
+      <c r="I102" s="27"/>
+      <c r="J102" s="55"/>
+      <c r="K102" s="56"/>
+      <c r="L102" s="56"/>
+      <c r="M102" s="55"/>
+      <c r="N102" s="91"/>
       <c r="O102" s="4"/>
     </row>
     <row r="103" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B103" s="27"/>
-      <c r="C103" s="28"/>
-      <c r="D103" s="28"/>
-      <c r="E103" s="28"/>
-      <c r="F103" s="26"/>
-      <c r="G103" s="27"/>
-      <c r="H103" s="28"/>
-      <c r="I103" s="26"/>
-      <c r="J103" s="22"/>
-      <c r="K103" s="23"/>
-      <c r="L103" s="23"/>
-      <c r="M103" s="22"/>
-      <c r="N103" s="24"/>
+      <c r="B103" s="25"/>
+      <c r="C103" s="26"/>
+      <c r="D103" s="26"/>
+      <c r="E103" s="26"/>
+      <c r="F103" s="27"/>
+      <c r="G103" s="25"/>
+      <c r="H103" s="26"/>
+      <c r="I103" s="27"/>
+      <c r="J103" s="55"/>
+      <c r="K103" s="56"/>
+      <c r="L103" s="56"/>
+      <c r="M103" s="55"/>
+      <c r="N103" s="91"/>
       <c r="O103" s="4"/>
     </row>
     <row r="104" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B104" s="27"/>
-      <c r="C104" s="28"/>
-      <c r="D104" s="28"/>
-      <c r="E104" s="28"/>
-      <c r="F104" s="26"/>
-      <c r="G104" s="27"/>
-      <c r="H104" s="28"/>
-      <c r="I104" s="26"/>
-      <c r="J104" s="22"/>
-      <c r="K104" s="23"/>
-      <c r="L104" s="23"/>
-      <c r="M104" s="22"/>
-      <c r="N104" s="24"/>
+      <c r="B104" s="25"/>
+      <c r="C104" s="26"/>
+      <c r="D104" s="26"/>
+      <c r="E104" s="26"/>
+      <c r="F104" s="27"/>
+      <c r="G104" s="25"/>
+      <c r="H104" s="26"/>
+      <c r="I104" s="27"/>
+      <c r="J104" s="55"/>
+      <c r="K104" s="56"/>
+      <c r="L104" s="56"/>
+      <c r="M104" s="55"/>
+      <c r="N104" s="91"/>
       <c r="O104" s="4"/>
     </row>
     <row r="105" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B105" s="27"/>
-      <c r="C105" s="28"/>
-      <c r="D105" s="28"/>
-      <c r="E105" s="28"/>
-      <c r="F105" s="26"/>
-      <c r="G105" s="27"/>
-      <c r="H105" s="28"/>
-      <c r="I105" s="26"/>
-      <c r="J105" s="22"/>
-      <c r="K105" s="23"/>
-      <c r="L105" s="23"/>
-      <c r="M105" s="22"/>
-      <c r="N105" s="24"/>
+      <c r="B105" s="25"/>
+      <c r="C105" s="26"/>
+      <c r="D105" s="26"/>
+      <c r="E105" s="26"/>
+      <c r="F105" s="27"/>
+      <c r="G105" s="25"/>
+      <c r="H105" s="26"/>
+      <c r="I105" s="27"/>
+      <c r="J105" s="55"/>
+      <c r="K105" s="56"/>
+      <c r="L105" s="56"/>
+      <c r="M105" s="55"/>
+      <c r="N105" s="91"/>
       <c r="O105" s="4"/>
     </row>
     <row r="106" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B106" s="27"/>
-      <c r="C106" s="28"/>
-      <c r="D106" s="28"/>
-      <c r="E106" s="28"/>
-      <c r="F106" s="26"/>
-      <c r="G106" s="27"/>
-      <c r="H106" s="28"/>
-      <c r="I106" s="26"/>
-      <c r="J106" s="22"/>
-      <c r="K106" s="23"/>
-      <c r="L106" s="23"/>
-      <c r="M106" s="22"/>
-      <c r="N106" s="24"/>
+      <c r="B106" s="25"/>
+      <c r="C106" s="26"/>
+      <c r="D106" s="26"/>
+      <c r="E106" s="26"/>
+      <c r="F106" s="27"/>
+      <c r="G106" s="25"/>
+      <c r="H106" s="26"/>
+      <c r="I106" s="27"/>
+      <c r="J106" s="55"/>
+      <c r="K106" s="56"/>
+      <c r="L106" s="56"/>
+      <c r="M106" s="55"/>
+      <c r="N106" s="91"/>
       <c r="O106" s="4"/>
     </row>
     <row r="107" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3912,120 +3912,120 @@
       <c r="O107" s="5"/>
     </row>
     <row r="108" spans="2:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B108" s="35" t="s">
+      <c r="B108" s="42" t="s">
         <v>165</v>
       </c>
-      <c r="C108" s="36"/>
-      <c r="D108" s="36"/>
-      <c r="E108" s="36"/>
-      <c r="F108" s="36"/>
-      <c r="G108" s="36"/>
-      <c r="H108" s="36"/>
-      <c r="I108" s="36"/>
-      <c r="J108" s="36"/>
-      <c r="K108" s="36"/>
-      <c r="L108" s="36"/>
-      <c r="M108" s="36"/>
-      <c r="N108" s="36"/>
-      <c r="O108" s="37"/>
+      <c r="C108" s="43"/>
+      <c r="D108" s="43"/>
+      <c r="E108" s="43"/>
+      <c r="F108" s="43"/>
+      <c r="G108" s="43"/>
+      <c r="H108" s="43"/>
+      <c r="I108" s="43"/>
+      <c r="J108" s="43"/>
+      <c r="K108" s="43"/>
+      <c r="L108" s="43"/>
+      <c r="M108" s="43"/>
+      <c r="N108" s="43"/>
+      <c r="O108" s="44"/>
     </row>
     <row r="109" spans="2:15" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B109" s="85" t="s">
+      <c r="B109" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="C109" s="28"/>
-      <c r="D109" s="28"/>
-      <c r="E109" s="28"/>
-      <c r="F109" s="28"/>
-      <c r="G109" s="28"/>
-      <c r="H109" s="28"/>
-      <c r="I109" s="28"/>
-      <c r="J109" s="28"/>
-      <c r="K109" s="28"/>
-      <c r="L109" s="28"/>
-      <c r="M109" s="28"/>
-      <c r="N109" s="28"/>
-      <c r="O109" s="26"/>
+      <c r="C109" s="26"/>
+      <c r="D109" s="26"/>
+      <c r="E109" s="26"/>
+      <c r="F109" s="26"/>
+      <c r="G109" s="26"/>
+      <c r="H109" s="26"/>
+      <c r="I109" s="26"/>
+      <c r="J109" s="26"/>
+      <c r="K109" s="26"/>
+      <c r="L109" s="26"/>
+      <c r="M109" s="26"/>
+      <c r="N109" s="26"/>
+      <c r="O109" s="27"/>
     </row>
     <row r="110" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B110" s="27"/>
-      <c r="C110" s="61"/>
-      <c r="D110" s="61"/>
-      <c r="E110" s="61"/>
-      <c r="F110" s="61"/>
-      <c r="G110" s="61"/>
-      <c r="H110" s="61"/>
-      <c r="I110" s="61"/>
-      <c r="J110" s="61"/>
-      <c r="K110" s="61"/>
-      <c r="L110" s="61"/>
-      <c r="M110" s="61"/>
-      <c r="N110" s="61"/>
-      <c r="O110" s="62"/>
+      <c r="B110" s="25"/>
+      <c r="C110" s="35"/>
+      <c r="D110" s="35"/>
+      <c r="E110" s="35"/>
+      <c r="F110" s="35"/>
+      <c r="G110" s="35"/>
+      <c r="H110" s="35"/>
+      <c r="I110" s="35"/>
+      <c r="J110" s="35"/>
+      <c r="K110" s="35"/>
+      <c r="L110" s="35"/>
+      <c r="M110" s="35"/>
+      <c r="N110" s="35"/>
+      <c r="O110" s="36"/>
     </row>
     <row r="111" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B111" s="70"/>
-      <c r="C111" s="71"/>
-      <c r="D111" s="71"/>
-      <c r="E111" s="71"/>
-      <c r="F111" s="71"/>
-      <c r="G111" s="71"/>
-      <c r="H111" s="71"/>
-      <c r="I111" s="71"/>
-      <c r="J111" s="71"/>
-      <c r="K111" s="71"/>
-      <c r="L111" s="71"/>
-      <c r="M111" s="71"/>
-      <c r="N111" s="71"/>
-      <c r="O111" s="72"/>
+      <c r="B111" s="47"/>
+      <c r="C111" s="51"/>
+      <c r="D111" s="51"/>
+      <c r="E111" s="51"/>
+      <c r="F111" s="51"/>
+      <c r="G111" s="51"/>
+      <c r="H111" s="51"/>
+      <c r="I111" s="51"/>
+      <c r="J111" s="51"/>
+      <c r="K111" s="51"/>
+      <c r="L111" s="51"/>
+      <c r="M111" s="51"/>
+      <c r="N111" s="51"/>
+      <c r="O111" s="48"/>
     </row>
     <row r="112" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B112" s="70"/>
-      <c r="C112" s="71"/>
-      <c r="D112" s="71"/>
-      <c r="E112" s="71"/>
-      <c r="F112" s="71"/>
-      <c r="G112" s="71"/>
-      <c r="H112" s="71"/>
-      <c r="I112" s="71"/>
-      <c r="J112" s="71"/>
-      <c r="K112" s="71"/>
-      <c r="L112" s="71"/>
-      <c r="M112" s="71"/>
-      <c r="N112" s="71"/>
-      <c r="O112" s="72"/>
+      <c r="B112" s="47"/>
+      <c r="C112" s="51"/>
+      <c r="D112" s="51"/>
+      <c r="E112" s="51"/>
+      <c r="F112" s="51"/>
+      <c r="G112" s="51"/>
+      <c r="H112" s="51"/>
+      <c r="I112" s="51"/>
+      <c r="J112" s="51"/>
+      <c r="K112" s="51"/>
+      <c r="L112" s="51"/>
+      <c r="M112" s="51"/>
+      <c r="N112" s="51"/>
+      <c r="O112" s="48"/>
     </row>
     <row r="113" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B113" s="70"/>
-      <c r="C113" s="71"/>
-      <c r="D113" s="71"/>
-      <c r="E113" s="71"/>
-      <c r="F113" s="71"/>
-      <c r="G113" s="71"/>
-      <c r="H113" s="71"/>
-      <c r="I113" s="71"/>
-      <c r="J113" s="71"/>
-      <c r="K113" s="71"/>
-      <c r="L113" s="71"/>
-      <c r="M113" s="71"/>
-      <c r="N113" s="71"/>
-      <c r="O113" s="72"/>
+      <c r="B113" s="47"/>
+      <c r="C113" s="51"/>
+      <c r="D113" s="51"/>
+      <c r="E113" s="51"/>
+      <c r="F113" s="51"/>
+      <c r="G113" s="51"/>
+      <c r="H113" s="51"/>
+      <c r="I113" s="51"/>
+      <c r="J113" s="51"/>
+      <c r="K113" s="51"/>
+      <c r="L113" s="51"/>
+      <c r="M113" s="51"/>
+      <c r="N113" s="51"/>
+      <c r="O113" s="48"/>
     </row>
     <row r="114" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B114" s="63"/>
-      <c r="C114" s="64"/>
-      <c r="D114" s="64"/>
-      <c r="E114" s="64"/>
-      <c r="F114" s="64"/>
-      <c r="G114" s="64"/>
-      <c r="H114" s="64"/>
-      <c r="I114" s="64"/>
-      <c r="J114" s="64"/>
-      <c r="K114" s="64"/>
-      <c r="L114" s="64"/>
-      <c r="M114" s="64"/>
-      <c r="N114" s="64"/>
-      <c r="O114" s="65"/>
+      <c r="B114" s="37"/>
+      <c r="C114" s="38"/>
+      <c r="D114" s="38"/>
+      <c r="E114" s="38"/>
+      <c r="F114" s="38"/>
+      <c r="G114" s="38"/>
+      <c r="H114" s="38"/>
+      <c r="I114" s="38"/>
+      <c r="J114" s="38"/>
+      <c r="K114" s="38"/>
+      <c r="L114" s="38"/>
+      <c r="M114" s="38"/>
+      <c r="N114" s="38"/>
+      <c r="O114" s="39"/>
     </row>
     <row r="115" spans="2:16" ht="16.5" x14ac:dyDescent="0.3">
       <c r="B115" s="9"/>
@@ -4044,154 +4044,363 @@
       <c r="O115" s="11"/>
     </row>
     <row r="116" spans="2:16" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B116" s="29" t="s">
+      <c r="B116" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="C116" s="30"/>
-      <c r="D116" s="30"/>
-      <c r="E116" s="30"/>
-      <c r="F116" s="30"/>
-      <c r="G116" s="30"/>
-      <c r="H116" s="31"/>
-      <c r="I116" s="29" t="s">
+      <c r="C116" s="85"/>
+      <c r="D116" s="85"/>
+      <c r="E116" s="85"/>
+      <c r="F116" s="85"/>
+      <c r="G116" s="85"/>
+      <c r="H116" s="86"/>
+      <c r="I116" s="87" t="s">
         <v>157</v>
       </c>
-      <c r="J116" s="30"/>
-      <c r="K116" s="30"/>
-      <c r="L116" s="30"/>
-      <c r="M116" s="30"/>
-      <c r="N116" s="30"/>
-      <c r="O116" s="34"/>
+      <c r="J116" s="85"/>
+      <c r="K116" s="85"/>
+      <c r="L116" s="85"/>
+      <c r="M116" s="85"/>
+      <c r="N116" s="85"/>
+      <c r="O116" s="88"/>
       <c r="P116" s="12"/>
     </row>
     <row r="117" spans="2:16" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="32" t="s">
+      <c r="B117" s="83" t="s">
         <v>123</v>
       </c>
-      <c r="C117" s="33"/>
-      <c r="D117" s="33"/>
-      <c r="E117" s="33"/>
-      <c r="F117" s="33"/>
-      <c r="G117" s="33"/>
-      <c r="H117" s="33"/>
-      <c r="I117" s="32" t="s">
+      <c r="C117" s="81"/>
+      <c r="D117" s="81"/>
+      <c r="E117" s="81"/>
+      <c r="F117" s="81"/>
+      <c r="G117" s="81"/>
+      <c r="H117" s="81"/>
+      <c r="I117" s="83" t="s">
         <v>123</v>
       </c>
-      <c r="J117" s="33"/>
-      <c r="K117" s="33"/>
-      <c r="L117" s="33"/>
-      <c r="M117" s="33"/>
-      <c r="N117" s="33"/>
-      <c r="O117" s="33"/>
+      <c r="J117" s="81"/>
+      <c r="K117" s="81"/>
+      <c r="L117" s="81"/>
+      <c r="M117" s="81"/>
+      <c r="N117" s="81"/>
+      <c r="O117" s="81"/>
       <c r="P117" s="12"/>
     </row>
     <row r="118" spans="2:16" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B118" s="54" t="s">
+      <c r="B118" s="50" t="s">
         <v>154</v>
       </c>
-      <c r="C118" s="28"/>
-      <c r="D118" s="28"/>
-      <c r="E118" s="26"/>
-      <c r="F118" s="54" t="s">
+      <c r="C118" s="26"/>
+      <c r="D118" s="26"/>
+      <c r="E118" s="27"/>
+      <c r="F118" s="50" t="s">
         <v>154</v>
       </c>
-      <c r="G118" s="28"/>
-      <c r="H118" s="28"/>
-      <c r="I118" s="28"/>
-      <c r="J118" s="26"/>
-      <c r="K118" s="54" t="s">
+      <c r="G118" s="26"/>
+      <c r="H118" s="26"/>
+      <c r="I118" s="26"/>
+      <c r="J118" s="27"/>
+      <c r="K118" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="L118" s="28"/>
-      <c r="M118" s="28"/>
-      <c r="N118" s="28"/>
-      <c r="O118" s="26"/>
+      <c r="L118" s="26"/>
+      <c r="M118" s="26"/>
+      <c r="N118" s="26"/>
+      <c r="O118" s="27"/>
     </row>
     <row r="119" spans="2:16" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B119" s="51" t="s">
+      <c r="B119" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="C119" s="52"/>
-      <c r="D119" s="52"/>
-      <c r="E119" s="53"/>
-      <c r="F119" s="51" t="s">
+      <c r="C119" s="53"/>
+      <c r="D119" s="53"/>
+      <c r="E119" s="54"/>
+      <c r="F119" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="G119" s="52"/>
-      <c r="H119" s="52"/>
-      <c r="I119" s="52"/>
-      <c r="J119" s="53"/>
-      <c r="K119" s="51" t="s">
+      <c r="G119" s="53"/>
+      <c r="H119" s="53"/>
+      <c r="I119" s="53"/>
+      <c r="J119" s="54"/>
+      <c r="K119" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="L119" s="52"/>
-      <c r="M119" s="52"/>
-      <c r="N119" s="52"/>
-      <c r="O119" s="53"/>
+      <c r="L119" s="53"/>
+      <c r="M119" s="53"/>
+      <c r="N119" s="53"/>
+      <c r="O119" s="54"/>
     </row>
     <row r="120" spans="2:16" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B120" s="41" t="s">
+      <c r="B120" s="73" t="s">
         <v>105</v>
       </c>
-      <c r="C120" s="36"/>
-      <c r="D120" s="36"/>
-      <c r="E120" s="36"/>
-      <c r="F120" s="36"/>
-      <c r="G120" s="36"/>
-      <c r="H120" s="36"/>
-      <c r="I120" s="36"/>
-      <c r="J120" s="36"/>
-      <c r="K120" s="36"/>
-      <c r="L120" s="36"/>
-      <c r="M120" s="36"/>
-      <c r="N120" s="36"/>
-      <c r="O120" s="37"/>
+      <c r="C120" s="43"/>
+      <c r="D120" s="43"/>
+      <c r="E120" s="43"/>
+      <c r="F120" s="43"/>
+      <c r="G120" s="43"/>
+      <c r="H120" s="43"/>
+      <c r="I120" s="43"/>
+      <c r="J120" s="43"/>
+      <c r="K120" s="43"/>
+      <c r="L120" s="43"/>
+      <c r="M120" s="43"/>
+      <c r="N120" s="43"/>
+      <c r="O120" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="324">
-    <mergeCell ref="F7:O7"/>
-    <mergeCell ref="F8:O8"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="E77:G77"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="N62:O62"/>
-    <mergeCell ref="N74:O74"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B92:E92"/>
-    <mergeCell ref="F94:G94"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="H93:M93"/>
-    <mergeCell ref="N72:O72"/>
-    <mergeCell ref="G102:I102"/>
-    <mergeCell ref="N63:O63"/>
-    <mergeCell ref="J101:L101"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="N68:O68"/>
-    <mergeCell ref="E66:G66"/>
-    <mergeCell ref="B95:E95"/>
-    <mergeCell ref="F93:G93"/>
-    <mergeCell ref="I15:O15"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="N92:O92"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="H62:J62"/>
-    <mergeCell ref="H46:K47"/>
-    <mergeCell ref="E67:G67"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="E62:G62"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="N69:O69"/>
-    <mergeCell ref="H75:J75"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B44:O44"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="B60:O60"/>
-    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="B100:O100"/>
+    <mergeCell ref="M101:N101"/>
+    <mergeCell ref="J105:L105"/>
+    <mergeCell ref="J106:L106"/>
+    <mergeCell ref="M102:N102"/>
+    <mergeCell ref="M103:N103"/>
+    <mergeCell ref="M104:N104"/>
+    <mergeCell ref="M105:N105"/>
+    <mergeCell ref="M106:N106"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="D86:I86"/>
+    <mergeCell ref="J86:L86"/>
+    <mergeCell ref="M86:O86"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="D87:I87"/>
+    <mergeCell ref="J87:L87"/>
+    <mergeCell ref="M87:O87"/>
+    <mergeCell ref="B88:C88"/>
+    <mergeCell ref="D88:I88"/>
+    <mergeCell ref="J88:L88"/>
+    <mergeCell ref="M88:O88"/>
+    <mergeCell ref="B24:O24"/>
+    <mergeCell ref="B117:H117"/>
+    <mergeCell ref="B116:H116"/>
+    <mergeCell ref="I116:O116"/>
+    <mergeCell ref="I117:O117"/>
+    <mergeCell ref="B83:O83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="D84:I84"/>
+    <mergeCell ref="J84:L84"/>
+    <mergeCell ref="M84:O84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="D85:I85"/>
+    <mergeCell ref="J85:L85"/>
+    <mergeCell ref="M85:O85"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="B33:O33"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="K34:O34"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="K25:O25"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="K39:L39"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:L38"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="B120:O120"/>
+    <mergeCell ref="B104:F104"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="B3:O3"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="E63:G63"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="N77:O77"/>
+    <mergeCell ref="N79:O79"/>
+    <mergeCell ref="N73:O73"/>
+    <mergeCell ref="H79:J79"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="J104:L104"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="I12:O12"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B119:E119"/>
+    <mergeCell ref="B102:F102"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="N71:O71"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="K119:O119"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H94:M94"/>
+    <mergeCell ref="F118:J118"/>
+    <mergeCell ref="B10:I10"/>
+    <mergeCell ref="H69:J69"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="I11:O11"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="E56:G56"/>
+    <mergeCell ref="B103:F103"/>
+    <mergeCell ref="B51:D52"/>
+    <mergeCell ref="E69:G69"/>
+    <mergeCell ref="H80:J80"/>
+    <mergeCell ref="B108:O108"/>
+    <mergeCell ref="B101:F101"/>
+    <mergeCell ref="G106:I106"/>
+    <mergeCell ref="L45:O45"/>
+    <mergeCell ref="H64:J64"/>
+    <mergeCell ref="N91:O91"/>
+    <mergeCell ref="B14:O14"/>
+    <mergeCell ref="H77:J77"/>
+    <mergeCell ref="E76:G76"/>
+    <mergeCell ref="E78:G78"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B43:O43"/>
+    <mergeCell ref="I16:O19"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="B49:O49"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="H71:J71"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="N64:O64"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="H56:K56"/>
+    <mergeCell ref="L56:O56"/>
+    <mergeCell ref="B57:D58"/>
+    <mergeCell ref="E57:G58"/>
+    <mergeCell ref="H57:K58"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="B16:H19"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B46:D47"/>
+    <mergeCell ref="N80:O80"/>
+    <mergeCell ref="J103:L103"/>
+    <mergeCell ref="N96:O96"/>
+    <mergeCell ref="N97:O97"/>
+    <mergeCell ref="H73:J73"/>
+    <mergeCell ref="F97:G97"/>
+    <mergeCell ref="E68:G68"/>
+    <mergeCell ref="B4:O4"/>
+    <mergeCell ref="H97:M97"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="N76:O76"/>
+    <mergeCell ref="B78:C81"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="L57:O58"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="H53:K53"/>
+    <mergeCell ref="L53:O53"/>
+    <mergeCell ref="B54:D55"/>
+    <mergeCell ref="E54:G55"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="N81:O81"/>
+    <mergeCell ref="H50:K50"/>
+    <mergeCell ref="N75:O75"/>
+    <mergeCell ref="L51:O52"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="J102:L102"/>
+    <mergeCell ref="E79:G79"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="N61:O61"/>
+    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="B62:C65"/>
+    <mergeCell ref="B66:C69"/>
+    <mergeCell ref="H96:M96"/>
+    <mergeCell ref="E51:G52"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="B23:O23"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="L20:O20"/>
+    <mergeCell ref="N67:O67"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="E74:G74"/>
+    <mergeCell ref="H54:K55"/>
+    <mergeCell ref="L54:O55"/>
+    <mergeCell ref="F119:J119"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="E71:G71"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="G105:I105"/>
+    <mergeCell ref="H76:J76"/>
+    <mergeCell ref="E80:G80"/>
+    <mergeCell ref="G104:I104"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="N65:O65"/>
+    <mergeCell ref="H92:M92"/>
+    <mergeCell ref="H81:J81"/>
+    <mergeCell ref="G101:I101"/>
+    <mergeCell ref="F96:G96"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="E73:G73"/>
+    <mergeCell ref="N93:O93"/>
+    <mergeCell ref="H67:J67"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="H91:M91"/>
+    <mergeCell ref="H74:J74"/>
+    <mergeCell ref="K118:O118"/>
+    <mergeCell ref="B105:F105"/>
+    <mergeCell ref="B110:O114"/>
+    <mergeCell ref="B99:O99"/>
+    <mergeCell ref="B118:E118"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="G103:I103"/>
+    <mergeCell ref="H72:J72"/>
+    <mergeCell ref="H66:J66"/>
+    <mergeCell ref="L50:O50"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H51:K52"/>
+    <mergeCell ref="E70:G70"/>
+    <mergeCell ref="E46:G47"/>
+    <mergeCell ref="N78:O78"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="E72:G72"/>
+    <mergeCell ref="L46:O47"/>
+    <mergeCell ref="H70:J70"/>
     <mergeCell ref="F92:G92"/>
     <mergeCell ref="L5:O5"/>
     <mergeCell ref="B109:O109"/>
@@ -4216,263 +4425,54 @@
     <mergeCell ref="E75:G75"/>
     <mergeCell ref="N95:O95"/>
     <mergeCell ref="F95:G95"/>
+    <mergeCell ref="B92:E92"/>
+    <mergeCell ref="F94:G94"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="H93:M93"/>
+    <mergeCell ref="N72:O72"/>
+    <mergeCell ref="G102:I102"/>
+    <mergeCell ref="N63:O63"/>
+    <mergeCell ref="J101:L101"/>
+    <mergeCell ref="N68:O68"/>
+    <mergeCell ref="E66:G66"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="F93:G93"/>
+    <mergeCell ref="N92:O92"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="H62:J62"/>
+    <mergeCell ref="H46:K47"/>
+    <mergeCell ref="E67:G67"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="N69:O69"/>
+    <mergeCell ref="H75:J75"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B44:O44"/>
+    <mergeCell ref="F7:O7"/>
+    <mergeCell ref="F8:O8"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="E77:G77"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="N62:O62"/>
+    <mergeCell ref="N74:O74"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="I15:O15"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="B60:O60"/>
+    <mergeCell ref="H21:K21"/>
     <mergeCell ref="H65:J65"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="K31:L31"/>
     <mergeCell ref="N66:O66"/>
     <mergeCell ref="B74:C77"/>
-    <mergeCell ref="H91:M91"/>
-    <mergeCell ref="H74:J74"/>
-    <mergeCell ref="K118:O118"/>
-    <mergeCell ref="B105:F105"/>
-    <mergeCell ref="B110:O114"/>
-    <mergeCell ref="B99:O99"/>
-    <mergeCell ref="B118:E118"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="G103:I103"/>
-    <mergeCell ref="H72:J72"/>
-    <mergeCell ref="H66:J66"/>
-    <mergeCell ref="L50:O50"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H51:K52"/>
-    <mergeCell ref="E70:G70"/>
-    <mergeCell ref="E46:G47"/>
-    <mergeCell ref="N78:O78"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="E72:G72"/>
-    <mergeCell ref="L46:O47"/>
-    <mergeCell ref="H70:J70"/>
-    <mergeCell ref="E74:G74"/>
-    <mergeCell ref="H54:K55"/>
-    <mergeCell ref="L54:O55"/>
-    <mergeCell ref="F119:J119"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="E71:G71"/>
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="G105:I105"/>
-    <mergeCell ref="H76:J76"/>
-    <mergeCell ref="E80:G80"/>
-    <mergeCell ref="G104:I104"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="N81:O81"/>
-    <mergeCell ref="H50:K50"/>
-    <mergeCell ref="N75:O75"/>
-    <mergeCell ref="L51:O52"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="J102:L102"/>
-    <mergeCell ref="E79:G79"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="N61:O61"/>
-    <mergeCell ref="B91:E91"/>
-    <mergeCell ref="B62:C65"/>
-    <mergeCell ref="B66:C69"/>
-    <mergeCell ref="H96:M96"/>
-    <mergeCell ref="E51:G52"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="B23:O23"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="N67:O67"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="N65:O65"/>
-    <mergeCell ref="B46:D47"/>
-    <mergeCell ref="N80:O80"/>
-    <mergeCell ref="J103:L103"/>
-    <mergeCell ref="N96:O96"/>
-    <mergeCell ref="N97:O97"/>
-    <mergeCell ref="H73:J73"/>
-    <mergeCell ref="F97:G97"/>
-    <mergeCell ref="E68:G68"/>
-    <mergeCell ref="B4:O4"/>
-    <mergeCell ref="H97:M97"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N76:O76"/>
-    <mergeCell ref="B78:C81"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="L57:O58"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="E53:G53"/>
-    <mergeCell ref="H53:K53"/>
-    <mergeCell ref="L53:O53"/>
-    <mergeCell ref="B54:D55"/>
-    <mergeCell ref="E54:G55"/>
-    <mergeCell ref="B14:O14"/>
-    <mergeCell ref="H77:J77"/>
-    <mergeCell ref="E76:G76"/>
-    <mergeCell ref="E78:G78"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B43:O43"/>
-    <mergeCell ref="I16:O19"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="B49:O49"/>
-    <mergeCell ref="H92:M92"/>
-    <mergeCell ref="H81:J81"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="H71:J71"/>
-    <mergeCell ref="G101:I101"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="N64:O64"/>
-    <mergeCell ref="F96:G96"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="H56:K56"/>
-    <mergeCell ref="L56:O56"/>
-    <mergeCell ref="B57:D58"/>
-    <mergeCell ref="E57:G58"/>
-    <mergeCell ref="H57:K58"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="B16:H19"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="E73:G73"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="N71:O71"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="K119:O119"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H94:M94"/>
-    <mergeCell ref="F118:J118"/>
-    <mergeCell ref="B10:I10"/>
-    <mergeCell ref="H69:J69"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="I11:O11"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="E56:G56"/>
-    <mergeCell ref="B103:F103"/>
-    <mergeCell ref="B51:D52"/>
-    <mergeCell ref="E69:G69"/>
-    <mergeCell ref="H80:J80"/>
-    <mergeCell ref="B108:O108"/>
-    <mergeCell ref="B101:F101"/>
-    <mergeCell ref="G106:I106"/>
-    <mergeCell ref="L45:O45"/>
-    <mergeCell ref="H64:J64"/>
-    <mergeCell ref="N91:O91"/>
-    <mergeCell ref="N93:O93"/>
-    <mergeCell ref="H67:J67"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="B120:O120"/>
-    <mergeCell ref="B104:F104"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="B3:O3"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="E63:G63"/>
-    <mergeCell ref="H45:K45"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="N77:O77"/>
-    <mergeCell ref="N79:O79"/>
-    <mergeCell ref="N73:O73"/>
-    <mergeCell ref="H79:J79"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="J104:L104"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="I12:O12"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B119:E119"/>
-    <mergeCell ref="B102:F102"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="K40:L40"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="K38:L38"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="K25:O25"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="K39:L39"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="B24:O24"/>
-    <mergeCell ref="B117:H117"/>
-    <mergeCell ref="B116:H116"/>
-    <mergeCell ref="I116:O116"/>
-    <mergeCell ref="I117:O117"/>
-    <mergeCell ref="B83:O83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="D84:I84"/>
-    <mergeCell ref="J84:L84"/>
-    <mergeCell ref="M84:O84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="D85:I85"/>
-    <mergeCell ref="J85:L85"/>
-    <mergeCell ref="M85:O85"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="B33:O33"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="K34:O34"/>
-    <mergeCell ref="B25:J25"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="D86:I86"/>
-    <mergeCell ref="J86:L86"/>
-    <mergeCell ref="M86:O86"/>
-    <mergeCell ref="B87:C87"/>
-    <mergeCell ref="D87:I87"/>
-    <mergeCell ref="J87:L87"/>
-    <mergeCell ref="M87:O87"/>
-    <mergeCell ref="B88:C88"/>
-    <mergeCell ref="D88:I88"/>
-    <mergeCell ref="J88:L88"/>
-    <mergeCell ref="M88:O88"/>
-    <mergeCell ref="B100:O100"/>
-    <mergeCell ref="M101:N101"/>
-    <mergeCell ref="J105:L105"/>
-    <mergeCell ref="J106:L106"/>
-    <mergeCell ref="M102:N102"/>
-    <mergeCell ref="M103:N103"/>
-    <mergeCell ref="M104:N104"/>
-    <mergeCell ref="M105:N105"/>
-    <mergeCell ref="M106:N106"/>
   </mergeCells>
   <conditionalFormatting sqref="D62:D82">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>